<commit_message>
add new ARB and PolyAudit suspects evidence
</commit_message>
<xml_diff>
--- a/Evidence Register.xlsx
+++ b/Evidence Register.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="781">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1687" uniqueCount="1002">
   <si>
     <t>Evidence ID</t>
   </si>
@@ -2474,6 +2474,669 @@
       </rPr>
       <t>https://d3ok4keidno21i.cloudfront.net/</t>
     </r>
+  </si>
+  <si>
+    <t>PM-STMT-001</t>
+  </si>
+  <si>
+    <t>Polymarket Statements</t>
+  </si>
+  <si>
+    <t>Screenshot 2026-06-23 032512.png</t>
+  </si>
+  <si>
+    <t>PM-STMT-001_2026-06-23_Polymarket_X_White_House_MOU_Aimed_Ending_Conflict.png</t>
+  </si>
+  <si>
+    <t>Screenshot of Polymarket X post stating: “JUST IN: White House announces Trump has officially signed the memorandum of understanding aimed at ending the conflict with Iran.” The screenshot also shows replies questioning the relationship between Polymarket’s post wording and the market resolution.</t>
+  </si>
+  <si>
+    <t>Polymarket X account, @Polymarket</t>
+  </si>
+  <si>
+    <t>Omer Kabir</t>
+  </si>
+  <si>
+    <t>2026-06-18 1:06 AM displayed by X, timezone requires verification</t>
+  </si>
+  <si>
+    <t>Displayed X/browser timezone, verify against permalink if preserved</t>
+  </si>
+  <si>
+    <t>Polymarket public statement after disputed YES resolution</t>
+  </si>
+  <si>
+    <t>High. Polymarket’s own wording describes the instrument as a memorandum of understanding aimed at ending the conflict, not as a completed permanent peace deal. Supports claimant position that the June 15 market criteria require strict review.</t>
+  </si>
+  <si>
+    <t>Screenshot preserved. Public permalink and web archive capture recommended.</t>
+  </si>
+  <si>
+    <t>Market Rules; Resolution Evidence; PM-NEW-001; UMA-001; ARB-001</t>
+  </si>
+  <si>
+    <t>ceb904385b333f2b9036ab1968eaabaff062f8c3b9d329ba94c4096685d99a51</t>
+  </si>
+  <si>
+    <t>Do not characterize as an admission without counsel. Use as Polymarket-originated contextual evidence showing contemporaneous wording around the MOU.</t>
+  </si>
+  <si>
+    <t>PM-STMT-002</t>
+  </si>
+  <si>
+    <t>Screenshot 2026-06-23 032537.png</t>
+  </si>
+  <si>
+    <t>PM-STMT-002_2026-06-23_Polymarket_X_Iranian_President_And_White_House_MOU_Posts.png</t>
+  </si>
+  <si>
+    <t>Screenshot of Polymarket X posts dated June 18. One post states that Iranian President Masoud Pezeshkian signs a memorandum of understanding. A quoted Polymarket post states that the White House announced Trump officially signed the memorandum of understanding aimed at ending the conflict with Iran.</t>
+  </si>
+  <si>
+    <t>2026-06-18, exact time only partially visible in screenshot</t>
+  </si>
+  <si>
+    <t>Polymarket public statements concerning the alleged MOU after disputed market resolution</t>
+  </si>
+  <si>
+    <t>High. Shows Polymarket publicly described both sides as signing a memorandum of understanding, supporting further review of whether the market’s written “permanent peace deal” requirement was actually met.</t>
+  </si>
+  <si>
+    <t>Screenshot preserved. Public permalinks and web archive captures recommended.</t>
+  </si>
+  <si>
+    <t>Market Rules; Resolution Evidence; PM-STMT-001; PM-NEW-001; UMA-001; ARB-001</t>
+  </si>
+  <si>
+    <t>43a648a1b5f8659fb044166246b7ac7c1226325619afab9d4aa6cd62aa89792d</t>
+  </si>
+  <si>
+    <t>Important distinction: an MOU aimed at ending conflict may support negotiations or framework evidence, but is not automatically the same thing as a permanent peace deal under the disputed market rules.</t>
+  </si>
+  <si>
+    <t>PM-NEW-001</t>
+  </si>
+  <si>
+    <t>Polymarket Statements / Market Rules</t>
+  </si>
+  <si>
+    <t>Screenshot_2026-06-22-22-44-37-55_de89569fcedd2ee7e089530771d25907.jpg</t>
+  </si>
+  <si>
+    <t>PM-NEW-001_2026-06-22_Polymarket_US_Iran_Final_Nuclear_Deal_Rules_Screenshot.jpg</t>
+  </si>
+  <si>
+    <t>Screenshot of later Polymarket market titled “US-Iran Final Nuclear Deal by...?” The visible rules state that on June 14, 2026, the United States and Iran announced a written diplomatic agreement including a 60-day extendable period in which both countries committed to negotiate toward a “final deal.”</t>
+  </si>
+  <si>
+    <t>Polymarket market page</t>
+  </si>
+  <si>
+    <t>Underlying market page visible on or around 2026-06-22</t>
+  </si>
+  <si>
+    <t>UTC / local device time should be verified</t>
+  </si>
+  <si>
+    <t>Later Polymarket market language concerning June 14 agreement and future final deal negotiations</t>
+  </si>
+  <si>
+    <t>Very High. Polymarket’s later market wording appears to describe the June 14 agreement as a negotiation framework toward a final deal, which is relevant to whether the earlier June 15 permanent peace deal market should have resolved YES.</t>
+  </si>
+  <si>
+    <t>Screenshot preserved. Full page PDF, URL, and archived copy recommended.</t>
+  </si>
+  <si>
+    <t>Market Rules; Resolution Evidence; PM-STMT-001; PM-STMT-002; UMA-001; ARB-001</t>
+  </si>
+  <si>
+    <t>1e3aabeea73d7e4ced1ee5f9a908967dc03073a69bfdcb5d8305859e58cb8d0a</t>
+  </si>
+  <si>
+    <t>Use as inconsistent-treatment or Polymarket-originated contextual evidence. Do not call it a legal admission unless counsel approves.</t>
+  </si>
+  <si>
+    <t>DR-001</t>
+  </si>
+  <si>
+    <t>Blockchain, wallet analysis, UMA vote</t>
+  </si>
+  <si>
+    <t>run_summary.json</t>
+  </si>
+  <si>
+    <t>DR-001_depth4_top12_uma_onchain_run_summary.json</t>
+  </si>
+  <si>
+    <t>Run summary for the focused depth-4 on-chain path analysis targeting Top 12 UMA whale staker or delegate addresses against 21 known Polymarket-side / conflict source wallets. The run used focused seed mode, excluded Top UMA whale targets from source wallets, hid exact-overlap leads, visited 500 on-chain addresses, and produced 21 path rows.</t>
+  </si>
+  <si>
+    <t>Generated by deep_uma_poly_relation_miner_v8b_resilient_transfers.py from public Polygon data and local evidence repository</t>
+  </si>
+  <si>
+    <t>UTC / Polygon</t>
+  </si>
+  <si>
+    <t>Top 12 UMA whale path test; relation mining</t>
+  </si>
+  <si>
+    <t>Documents the methodology and limits of the focused depth-4 path test. Important because the test did not prove a strong Top 12 UMA whale connection after review, but did produce candidate paths and supporting relation data.</t>
+  </si>
+  <si>
+    <t>Derived analysis, methodologically useful; requires manual review of each path edge</t>
+  </si>
+  <si>
+    <t>UMA-WHALE-001; UMA-VAL-001; APP-CONFLICT-001; ARB-001</t>
+  </si>
+  <si>
+    <t>e3b9e12150b34319067e3b0870845fc4d430b24f9706c782c75f2341855189a3</t>
+  </si>
+  <si>
+    <t>Key metrics: 24 UMA target addresses, 21 Polymarket source addresses, 45 seed addresses, 920,396 edges, 47,008 nodes, 21 path rows, 12 clusters. The later review found most Top 12 paths passed through spam-token or generic-contract edges and should not be treated as strong linkage evidence.</t>
+  </si>
+  <si>
+    <t>DR-002</t>
+  </si>
+  <si>
+    <t>paths_to_uma_vote.csv</t>
+  </si>
+  <si>
+    <t>DR-002_depth4_top12_uma_paths_to_vote.csv</t>
+  </si>
+  <si>
+    <t>Candidate path output from the focused depth-4 run. It records 21 paths from known Polymarket-side / conflict wallets toward Top 12 UMA whale target addresses after exact-overlap rows were hidden.</t>
+  </si>
+  <si>
+    <t>Top 12 UMA whale path test</t>
+  </si>
+  <si>
+    <t>Useful as a negative or cautionary result. The output shows candidate paths, but manual review indicates most Top 12 paths route through spam-token or generic-contract edges, especially 0x6f8a064... and the USDC contract 0x3c499c..., so it does not currently establish a strong Top 12 UMA whale connection.</t>
+  </si>
+  <si>
+    <t>Derived lead file; reviewed and mostly weak/noisy for Top 12 UMA linkage</t>
+  </si>
+  <si>
+    <t>DR-001; DR-003; DR-004; UMA-WHALE-001; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>5ad927234221948b8ea9959d4f5f5309f20d1a50c5b04f5aad0fef613b663c91</t>
+  </si>
+  <si>
+    <t>21 path rows. Review notes: 20 paths appear to involve spam-token or dust bridge 0x6f8a064..., and 1 path appears to involve Polygon USDC contract 0x3c499c..., which should not be used as ownership or coordination evidence without further support.</t>
+  </si>
+  <si>
+    <t>DR-003</t>
+  </si>
+  <si>
+    <t>high_priority_leads.csv</t>
+  </si>
+  <si>
+    <t>DR-003_depth4_top12_uma_high_priority_leads.csv</t>
+  </si>
+  <si>
+    <t>High-priority lead output corresponding to the 21 path rows from the depth-4 Top 12 UMA whale focused run.</t>
+  </si>
+  <si>
+    <t>Preserves the script-ranked leads for manual review. Subsequent analysis indicates the label 'high priority' should be treated as computational ranking only, not legal strength, because many paths rely on noisy spam-token or generic-contract edges.</t>
+  </si>
+  <si>
+    <t>Derived lead file; requires manual transaction-level review</t>
+  </si>
+  <si>
+    <t>DR-001; DR-002; DR-004; UMA-WHALE-001</t>
+  </si>
+  <si>
+    <t>Use carefully. Do not describe this file as proving Top UMA whale coordination. It is mainly a path triage file.</t>
+  </si>
+  <si>
+    <t>DR-004</t>
+  </si>
+  <si>
+    <t>Blockchain, wallet analysis</t>
+  </si>
+  <si>
+    <t>edges_key_targets.csv</t>
+  </si>
+  <si>
+    <t>DR-004_depth4_key_target_edges.csv</t>
+  </si>
+  <si>
+    <t>Key target edge extract from the depth-4 run, used to inspect the specific edges supporting candidate paths and to identify spam-token or generic-contract noise.</t>
+  </si>
+  <si>
+    <t>Top 12 UMA whale path test; edge verification</t>
+  </si>
+  <si>
+    <t>Important because it explains why the 21 Top 12 UMA path rows are currently weak: many supporting edges involve spam-token assets or generic contracts rather than meaningful funding, position transfer, resolver, or proposer relationships.</t>
+  </si>
+  <si>
+    <t>Derived analysis; useful for filtering false positives</t>
+  </si>
+  <si>
+    <t>DR-001; DR-002; DR-003; UMA-WHALE-001</t>
+  </si>
+  <si>
+    <t>8259018c8edb20bcceb7960c55fe350d7cd49fc4c85786706cfcca18b445a423</t>
+  </si>
+  <si>
+    <t>Used to support manual conclusion that the Top 12 UMA whale direct linkage theory is not currently proven by this run.</t>
+  </si>
+  <si>
+    <t>DR-005</t>
+  </si>
+  <si>
+    <t>acff_full_edges.csv</t>
+  </si>
+  <si>
+    <t>DR-005_depth4_acff32_full_edges.csv</t>
+  </si>
+  <si>
+    <t>Full edge extract involving 0xacff32..., a recurring activator / infrastructure lead seen around multiple known YES-side or suspect wallets.</t>
+  </si>
+  <si>
+    <t>Infrastructure / activator wallet review</t>
+  </si>
+  <si>
+    <t>Supports a moderate lead that 0xacff32... may be an infrastructure, activation, relayer, or operational wallet interacting with several relevant wallets. Many rows are zero-value native transactions, so this should not be framed as confirmed funding.</t>
+  </si>
+  <si>
+    <t>Derived lead file; moderate relevance, needs transaction purpose review</t>
+  </si>
+  <si>
+    <t>DR-001; SUS-006; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>5c107ea81b84394a42e6aefb7f834437ea9ae8a72b098da908b4477cd1f3993e</t>
+  </si>
+  <si>
+    <t>Use as an infrastructure lead only. Do not call 0xacff32... a common funder unless non-zero funding transactions are separately verified.</t>
+  </si>
+  <si>
+    <t>DR-006</t>
+  </si>
+  <si>
+    <t>top_uma_whale_focus_targets.csv</t>
+  </si>
+  <si>
+    <t>DR-006_depth4_top12_uma_focus_targets.csv</t>
+  </si>
+  <si>
+    <t>List of Top 12 UMA whale focus target addresses used by the depth-4 run, including staker and delegate / hot wallet addresses selected from Top_60_Whales.csv.</t>
+  </si>
+  <si>
+    <t>Generated from UMA-WHALE-001 Top_60_Whales.csv</t>
+  </si>
+  <si>
+    <t>Top 12 UMA whale target definition</t>
+  </si>
+  <si>
+    <t>Shows which UMA whale addresses were treated as targets in the focused depth-4 path test. This is important because proposer wallets such as 0xc337... and 0x5276... were not Top 12 UMA whale targets unless separately included.</t>
+  </si>
+  <si>
+    <t>Derived target list; verified against input file by script</t>
+  </si>
+  <si>
+    <t>UMA-WHALE-001; DR-001</t>
+  </si>
+  <si>
+    <t>38fed305113d233e611c522f176a7fa207c0391935b4131890ee3ae1afb1d59e</t>
+  </si>
+  <si>
+    <t>Use to clarify that the depth-4 run tested Top UMA whale voting addresses, not all UMA proposers, disputers, or resolver wallets.</t>
+  </si>
+  <si>
+    <t>DR-007</t>
+  </si>
+  <si>
+    <t>cluster_summary.csv; nodes.csv</t>
+  </si>
+  <si>
+    <t>DR-007_depth4_cluster_summary_and_nodes.csv</t>
+  </si>
+  <si>
+    <t>Cluster summary and node output from the focused depth-4 run. The run generated 12 clusters and 47,008 nodes after on-chain expansion.</t>
+  </si>
+  <si>
+    <t>Top 12 UMA whale path test; graph context</t>
+  </si>
+  <si>
+    <t>Provides graph context for the depth-4 run. It is useful for methodology and reproducibility, but should not be treated as proof of common ownership without edge-level review.</t>
+  </si>
+  <si>
+    <t>Derived graph context; requires edge-level review</t>
+  </si>
+  <si>
+    <t>DR-001; DR-002; DR-004</t>
+  </si>
+  <si>
+    <t>cluster_summary.csv=12ce430b11a14839520e312dfa7364234ea75893212b01999dfcb071596e2bf0; nodes.csv=79c66795348e11fb6950d31bbc5ce03aa877fa0d484ca9b0756ee39c322dcb17</t>
+  </si>
+  <si>
+    <t>Hash field contains both hashes because this is a combined graph-context row. If preferred, split into two separate register rows.</t>
+  </si>
+  <si>
+    <t>SUS-001</t>
+  </si>
+  <si>
+    <t>Blockchain, wallet analysis, PolyAudit conflict</t>
+  </si>
+  <si>
+    <t>00_tracked_wallets.csv</t>
+  </si>
+  <si>
+    <t>SUS-001_polyaudit_suspect_tracked_wallets.csv</t>
+  </si>
+  <si>
+    <t>Tracked wallet list used by the PolyAudit suspect deep profiler, including ARB, tf2, GroyperFinance, secretscent, RockSolidBond, key funders, intermediaries, UMA proposers, and protocol addresses.</t>
+  </si>
+  <si>
+    <t>Generated by poly_audit_suspect_deep_profiler.py from local evidence labels and public Polygon data</t>
+  </si>
+  <si>
+    <t>PolyAudit suspect profiler; target definition</t>
+  </si>
+  <si>
+    <t>Defines the wallets and labels used for the suspect-focused run. Important for reproducibility and for distinguishing source wallets, funders, intermediaries, protocol contracts, and UMA proposer leads.</t>
+  </si>
+  <si>
+    <t>Derived target list; useful for reproducibility</t>
+  </si>
+  <si>
+    <t>APP-CONFLICT-001; ARB-001; UMA-WHALE-001</t>
+  </si>
+  <si>
+    <t>7a4cfaa2001dfbee4d10fb2e5c3001b2fa522065a6218aff6581a2d24e1ea828</t>
+  </si>
+  <si>
+    <t>This file is a target list, not proof by itself.</t>
+  </si>
+  <si>
+    <t>SUS-002</t>
+  </si>
+  <si>
+    <t>01_all_suspect_transfers.csv; raw_asset_transfers.jsonl</t>
+  </si>
+  <si>
+    <t>SUS-002_all_suspect_transfers_and_raw_asset_transfers</t>
+  </si>
+  <si>
+    <t>Collected Polygon asset-transfer records for tracked suspect wallets and related addresses during the April 1 through June 21, 2026 review period.</t>
+  </si>
+  <si>
+    <t>Generated by poly_audit_suspect_deep_profiler.py using public Polygon / Alchemy asset transfer data</t>
+  </si>
+  <si>
+    <t>Suspect wallet transfer collection</t>
+  </si>
+  <si>
+    <t>Primary raw/flat transfer collection supporting the ARB to tf2, c417 funding, GroyperFinance, secretscent / RockSolidBond, acff32, and CTF transfer review outputs.</t>
+  </si>
+  <si>
+    <t>Derived on-chain extraction; high relevance as supporting data</t>
+  </si>
+  <si>
+    <t>SUS-001; SUS-003; SUS-004; SUS-005; SUS-006; SUS-007; SUS-008; SUS-009</t>
+  </si>
+  <si>
+    <t>01_all_suspect_transfers.csv=62015dea383cd913cfc7b0bae8f6286a6ded1d480e6b59e5cf831510ef2b5db7; raw_asset_transfers.jsonl=64be36e4d6355b213df4ecb5c672005d3ff6be0218a7c30d44be3d6117928687</t>
+  </si>
+  <si>
+    <t>Hash field contains both hashes because this row preserves the flat CSV and raw JSONL source output. The run had a late pandas trade-row parsing error, but transfer collection completed and these files were written before the crash.</t>
+  </si>
+  <si>
+    <t>SUS-003</t>
+  </si>
+  <si>
+    <t>02_direct_suspect_relations.csv</t>
+  </si>
+  <si>
+    <t>SUS-003_direct_suspect_relations.csv</t>
+  </si>
+  <si>
+    <t>Aggregated direct relation table between tracked suspect wallets, funders, UMA proposer leads, and known protocol addresses.</t>
+  </si>
+  <si>
+    <t>Generated by poly_audit_suspect_deep_profiler.py from public Polygon transfer data</t>
+  </si>
+  <si>
+    <t>Direct suspect relation review</t>
+  </si>
+  <si>
+    <t>Summarizes direct transfer relationships among tracked addresses. Useful for quickly identifying meaningful one-hop relationships such as protocol interactions, funder flows, and suspect-to-suspect transfers.</t>
+  </si>
+  <si>
+    <t>Derived analysis; high relevance for triage</t>
+  </si>
+  <si>
+    <t>SUS-001; SUS-002; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>d4ceb146c5f0adc57bbe668e85920949bca0605a6654a66837753f11f9894668</t>
+  </si>
+  <si>
+    <t>Contains 82 direct relation rows. Must be reviewed at transaction level before making legal claims.</t>
+  </si>
+  <si>
+    <t>SUS-004</t>
+  </si>
+  <si>
+    <t>03_arb_tf2_direct_relation.csv</t>
+  </si>
+  <si>
+    <t>SUS-004_arb_tf2_direct_relation.csv</t>
+  </si>
+  <si>
+    <t>Direct transfer evidence between ARB / ArmageddonRewardsBilly wallet 0xc8ab97... and tf2 wallet 0xa102b4..., including USDC.e, pUSD, and CTF / ERC1155 transfer rows.</t>
+  </si>
+  <si>
+    <t>ARB to tf2 direct relationship; conflict inquiry</t>
+  </si>
+  <si>
+    <t>Strong investigative lead because ARB and tf2 are both independently relevant to the Polymarket / UMA conflict analysis. The file shows repeated bilateral transfers before the disputed resolution.</t>
+  </si>
+  <si>
+    <t>Derived on-chain lead; strong, requires market-level token ID mapping</t>
+  </si>
+  <si>
+    <t>ARB-001; APP-CONFLICT-001; SUS-002; SUS-009</t>
+  </si>
+  <si>
+    <t>6092025c02e12c7d4730d0ab726ca84c3ebd1e21b1a9927386ff12a84a8f79a8</t>
+  </si>
+  <si>
+    <t>Contains 11 direct rows. Aggregate review shows tf2 to ARB: 100,000 USDC.e and 200,000 pUSD, plus CTF / ERC1155 rows; ARB to tf2: about 280,571 pUSD plus CTF / ERC1155 rows. Legal conclusion requires mapping CTF token IDs to the relevant market(s).</t>
+  </si>
+  <si>
+    <t>SUS-005</t>
+  </si>
+  <si>
+    <t>04_c417_funding_cluster.csv</t>
+  </si>
+  <si>
+    <t>SUS-005_c417_funding_cluster.csv</t>
+  </si>
+  <si>
+    <t>Funding-cluster output showing address 0xc417fd8e9661c0d2120b64a04bb3278c17e99db1 as a major USDC.e source for multiple YES-side or investigation-relevant wallets.</t>
+  </si>
+  <si>
+    <t>Shared funding network; YES-side wallet cluster</t>
+  </si>
+  <si>
+    <t>Strong funding-cluster lead. The file indicates 0xc417fd... funded multiple known suspect / YES-side wallets, including Shirtybonds, RockSolidBond, secretscent, GroyperFinance, Anghkooey, 0x52e5..., tf2, and Dripx.</t>
+  </si>
+  <si>
+    <t>Derived on-chain funding lead; strong, requires trade-timestamp comparison</t>
+  </si>
+  <si>
+    <t>APP-CONFLICT-001; SUS-002; SUS-004; SUS-007; SUS-008</t>
+  </si>
+  <si>
+    <t>a692394ba21f17453d20b2ddbb3c104cd145c682cadefdca51516ad80f12880f</t>
+  </si>
+  <si>
+    <t>Aggregate examples: Shirtybonds about 6.05M USDC.e, RockSolidBond about 3.50M USDC.e, secretscent about 2.48M USDC.e, GroyperFinance about 1.21M USDC.e, Anghkooey about 432k USDC.e, 0x52e5 about 276.7k USDC.e, tf2 about 103.4k USDC.e, Dripx about 60k USDC.e. Compare arrival times to Polymarket YES purchases.</t>
+  </si>
+  <si>
+    <t>SUS-006</t>
+  </si>
+  <si>
+    <t>05_acff32_activity_review.csv</t>
+  </si>
+  <si>
+    <t>SUS-006_acff32_activity_review.csv</t>
+  </si>
+  <si>
+    <t>Activity review for 0xacff32f36054e039003c7925f7834360531f1f9a, a recurring activator / infrastructure lead interacting with multiple relevant wallets.</t>
+  </si>
+  <si>
+    <t>Moderate lead. The address recurs around ARB, debased, HolyMoses7, RockSolidBond, yungstalin, JAHODA, 0x665d, secretscent, and GroyperFinance, but many rows are zero-value MATIC calls and should not be characterized as funding without further review.</t>
+  </si>
+  <si>
+    <t>Derived lead file; moderate relevance</t>
+  </si>
+  <si>
+    <t>DR-005; SUS-002; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>67724e39557adac4c760e2080e57519572e882a439bd4baa6b62a33670d93961</t>
+  </si>
+  <si>
+    <t>Contains 1293 rows. Approximately 1108 rows are zero-value MATIC calls. Use as possible activator / infrastructure lead, not confirmed funding evidence.</t>
+  </si>
+  <si>
+    <t>SUS-007</t>
+  </si>
+  <si>
+    <t>Blockchain, wallet analysis, UMA oracle, PolyAudit conflict</t>
+  </si>
+  <si>
+    <t>06_groyperfinance_profile.csv</t>
+  </si>
+  <si>
+    <t>SUS-007_groyperfinance_profile.csv</t>
+  </si>
+  <si>
+    <t>GroyperFinance-focused transfer and protocol-interaction profile. It shows GroyperFinance funded by 0xc417fd... and interacting with UMA OOv2 and UMA bond infrastructure.</t>
+  </si>
+  <si>
+    <t>GroyperFinance conflict inquiry; UMA proposer / oracle activity</t>
+  </si>
+  <si>
+    <t>Strong to moderate conflict lead because GroyperFinance appears both financially linked to the shared funding network and active around UMA oracle / bond contracts.</t>
+  </si>
+  <si>
+    <t>Derived on-chain profile; high relevance, requires receipt-level transaction review</t>
+  </si>
+  <si>
+    <t>APP-CONFLICT-001; SUS-002; SUS-003; SUS-005; UMA-VAL-001</t>
+  </si>
+  <si>
+    <t>f57270a4ed5d62963c8c3201a51dff693b345a9fe741f2296dfd69101173ec40</t>
+  </si>
+  <si>
+    <t>Aggregate review: 0xc417fd... to GroyperFinance about 1,205,486.15 USDC.e; GroyperFinance to UMA bond contract about 4,500 USDC.e; UMA bond contract to GroyperFinance about 4,000 USDC.e; GroyperFinance to UMA OOv2 about 750 USDC.e; UMA OOv2 to GroyperFinance about 1,000 USDC.e.</t>
+  </si>
+  <si>
+    <t>SUS-008</t>
+  </si>
+  <si>
+    <t>07_secretscent_rocksolid_profile.csv</t>
+  </si>
+  <si>
+    <t>SUS-008_secretscent_rocksolid_profile.csv</t>
+  </si>
+  <si>
+    <t>Profile of secretscent, RockSolidBond, reported intermediaries 0x245b... and 0xa4fc..., shared funder 0xc417fd..., and UMA proposer lead 0xc33780d8....</t>
+  </si>
+  <si>
+    <t>secretscent / RockSolidBond / UMA proposer connection inquiry</t>
+  </si>
+  <si>
+    <t>Strong to moderate lead. Shows large USDC.e flows among secretscent, RockSolidBond, their intermediaries, shared funder 0xc417fd..., and UMA proposer 0xc337..., supporting a focused conflict and funding-network inquiry.</t>
+  </si>
+  <si>
+    <t>Derived on-chain profile; high relevance, requires transaction-level review</t>
+  </si>
+  <si>
+    <t>APP-CONFLICT-001; SUS-002; SUS-005; UMA-VAL-001</t>
+  </si>
+  <si>
+    <t>929f91fe0fc4431bf1913484a91533d25a80b9513cfb2473e00a576a941bb501</t>
+  </si>
+  <si>
+    <t>Aggregate examples: 0xc417fd... to secretscent about 2,476,082.34 USDC.e; 0xc417fd... to RockSolidBond about 3,495,215.34 USDC.e; secretscent to RockSolidBond about 4,950,136.69 USDC.e; 0x245b intermediary to UMA proposer 0xc337 about 436,448 USDC.e; 0xc337 back to 0x245b about 221,232 USDC.e; 0xa4fc intermediary to 0xc337 about 106,500 USDC.e; 0xc337 back to 0xa4fc about 53,362 USDC.e.</t>
+  </si>
+  <si>
+    <t>SUS-009</t>
+  </si>
+  <si>
+    <t>Blockchain, token movement, PolyAudit conflict</t>
+  </si>
+  <si>
+    <t>08_ctf_erc1155_transfer_review.csv</t>
+  </si>
+  <si>
+    <t>SUS-009_ctf_erc1155_transfer_review.csv</t>
+  </si>
+  <si>
+    <t>CTF / ERC1155 position-transfer review for tracked suspect wallets. Rows require token-ID mapping to determine whether transfers relate to the US-Iran market or other Polymarket markets.</t>
+  </si>
+  <si>
+    <t>Generated by poly_audit_suspect_deep_profiler.py from public Polygon ERC1155 transfer data</t>
+  </si>
+  <si>
+    <t>CTF / ERC1155 token movement review</t>
+  </si>
+  <si>
+    <t>Useful for verifying whether ARB, tf2, rdba, and other tracked wallets transferred Polymarket outcome tokens between each other or through related addresses. It is not final market-specific proof until token IDs are mapped to condition IDs.</t>
+  </si>
+  <si>
+    <t>Derived token-movement lead; requires token-ID mapping</t>
+  </si>
+  <si>
+    <t>SUS-004; SUS-002; ARB-001; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>77deffb9e55c0e3b2a7563bb0ee671281e75dba6b40725c49abe1912a82015fb</t>
+  </si>
+  <si>
+    <t>Contains 10355 ERC1155 / CTF review rows. Next step is mapping token IDs to market condition IDs and identifying which rows relate to the June 15 market.</t>
+  </si>
+  <si>
+    <t>SUS-010</t>
+  </si>
+  <si>
+    <t>Analysis summary, PolyAudit conflict</t>
+  </si>
+  <si>
+    <t>poly_audit_suspect_findings_review_summary.csv</t>
+  </si>
+  <si>
+    <t>SUS-010_polyaudit_suspect_findings_review_summary.csv</t>
+  </si>
+  <si>
+    <t>Short review summary of the suspect-profiler outputs, ranking the main findings and separating strong leads from weaker / noisy leads.</t>
+  </si>
+  <si>
+    <t>Generated from review of SUS-001 through SUS-009</t>
+  </si>
+  <si>
+    <t>Suspect profiler review summary</t>
+  </si>
+  <si>
+    <t>Provides counsel-facing summary of the new findings: ARB to tf2 direct relationship, 0xc417fd... shared funding network, GroyperFinance oracle/funding profile, secretscent / RockSolidBond / 0xc337 network, and acff32 as a moderate infrastructure lead.</t>
+  </si>
+  <si>
+    <t>Derived summary; should be checked against underlying CSVs</t>
+  </si>
+  <si>
+    <t>SUS-001; SUS-002; SUS-003; SUS-004; SUS-005; SUS-006; SUS-007; SUS-008; SUS-009</t>
+  </si>
+  <si>
+    <t>71c8b4c3446f9ca6cef9e4480bc8c95c55bdf12a5f55475be7276112536cfecb</t>
+  </si>
+  <si>
+    <t>Use as an orientation note only. The underlying CSVs and transaction hashes remain the primary evidence.</t>
   </si>
 </sst>
 </file>
@@ -2654,7 +3317,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:S986" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:S984" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="19">
     <tableColumn name="Evidence ID" id="1"/>
     <tableColumn name="Evidence category" id="2"/>
@@ -7841,464 +8504,1184 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="15"/>
-      <c r="B85" s="16"/>
-      <c r="C85" s="16"/>
-      <c r="D85" s="16"/>
-      <c r="E85" s="11"/>
-      <c r="F85" s="11"/>
-      <c r="G85" s="16"/>
-      <c r="H85" s="16"/>
-      <c r="I85" s="11"/>
-      <c r="J85" s="11"/>
-      <c r="K85" s="11"/>
-      <c r="L85" s="16"/>
-      <c r="M85" s="11"/>
-      <c r="N85" s="11"/>
-      <c r="O85" s="11"/>
-      <c r="P85" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q85" s="11"/>
-      <c r="R85" s="11"/>
-      <c r="S85" s="11"/>
+      <c r="A85" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>782</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>784</v>
+      </c>
+      <c r="E85" s="8" t="s">
+        <v>785</v>
+      </c>
+      <c r="F85" s="8" t="s">
+        <v>786</v>
+      </c>
+      <c r="G85" s="7" t="s">
+        <v>787</v>
+      </c>
+      <c r="H85" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I85" s="8" t="s">
+        <v>788</v>
+      </c>
+      <c r="J85" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K85" s="8" t="s">
+        <v>789</v>
+      </c>
+      <c r="L85" s="7" t="s">
+        <v>790</v>
+      </c>
+      <c r="M85" s="8" t="s">
+        <v>791</v>
+      </c>
+      <c r="N85" s="8" t="s">
+        <v>792</v>
+      </c>
+      <c r="O85" s="8" t="s">
+        <v>793</v>
+      </c>
+      <c r="P85" s="8" t="s">
+        <v>745</v>
+      </c>
+      <c r="Q85" s="8" t="s">
+        <v>794</v>
+      </c>
+      <c r="R85" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S85" s="8" t="s">
+        <v>795</v>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="15"/>
-      <c r="B86" s="16"/>
-      <c r="C86" s="16"/>
-      <c r="D86" s="16"/>
-      <c r="E86" s="11"/>
-      <c r="F86" s="11"/>
-      <c r="G86" s="16"/>
-      <c r="H86" s="16"/>
-      <c r="I86" s="11"/>
-      <c r="J86" s="11"/>
-      <c r="K86" s="11"/>
-      <c r="L86" s="16"/>
-      <c r="M86" s="11"/>
-      <c r="N86" s="11"/>
-      <c r="O86" s="11"/>
-      <c r="P86" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q86" s="11"/>
-      <c r="R86" s="11"/>
-      <c r="S86" s="11"/>
+      <c r="A86" s="4" t="s">
+        <v>796</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>782</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>797</v>
+      </c>
+      <c r="D86" s="7" t="s">
+        <v>798</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>799</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>786</v>
+      </c>
+      <c r="G86" s="7" t="s">
+        <v>787</v>
+      </c>
+      <c r="H86" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I86" s="8" t="s">
+        <v>800</v>
+      </c>
+      <c r="J86" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K86" s="8" t="s">
+        <v>789</v>
+      </c>
+      <c r="L86" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="M86" s="8" t="s">
+        <v>802</v>
+      </c>
+      <c r="N86" s="8" t="s">
+        <v>803</v>
+      </c>
+      <c r="O86" s="8" t="s">
+        <v>804</v>
+      </c>
+      <c r="P86" s="8" t="s">
+        <v>745</v>
+      </c>
+      <c r="Q86" s="8" t="s">
+        <v>805</v>
+      </c>
+      <c r="R86" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S86" s="8" t="s">
+        <v>806</v>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="15"/>
-      <c r="B87" s="16"/>
-      <c r="C87" s="16"/>
-      <c r="D87" s="16"/>
-      <c r="E87" s="11"/>
-      <c r="F87" s="11"/>
-      <c r="G87" s="16"/>
-      <c r="H87" s="16"/>
-      <c r="I87" s="11"/>
-      <c r="J87" s="11"/>
-      <c r="K87" s="11"/>
-      <c r="L87" s="16"/>
-      <c r="M87" s="11"/>
-      <c r="N87" s="11"/>
-      <c r="O87" s="11"/>
-      <c r="P87" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q87" s="11"/>
-      <c r="R87" s="11"/>
-      <c r="S87" s="11"/>
+      <c r="A87" s="4" t="s">
+        <v>807</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>808</v>
+      </c>
+      <c r="C87" s="7" t="s">
+        <v>809</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>810</v>
+      </c>
+      <c r="E87" s="8" t="s">
+        <v>811</v>
+      </c>
+      <c r="F87" s="8" t="s">
+        <v>812</v>
+      </c>
+      <c r="G87" s="7" t="s">
+        <v>787</v>
+      </c>
+      <c r="H87" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I87" s="8" t="s">
+        <v>813</v>
+      </c>
+      <c r="J87" s="14">
+        <v>46195.0</v>
+      </c>
+      <c r="K87" s="8" t="s">
+        <v>814</v>
+      </c>
+      <c r="L87" s="7" t="s">
+        <v>815</v>
+      </c>
+      <c r="M87" s="8" t="s">
+        <v>816</v>
+      </c>
+      <c r="N87" s="8" t="s">
+        <v>817</v>
+      </c>
+      <c r="O87" s="8" t="s">
+        <v>818</v>
+      </c>
+      <c r="P87" s="8" t="s">
+        <v>745</v>
+      </c>
+      <c r="Q87" s="8" t="s">
+        <v>819</v>
+      </c>
+      <c r="R87" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S87" s="8" t="s">
+        <v>820</v>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="15"/>
-      <c r="B88" s="16"/>
-      <c r="C88" s="16"/>
-      <c r="D88" s="16"/>
-      <c r="E88" s="11"/>
-      <c r="F88" s="11"/>
-      <c r="G88" s="16"/>
-      <c r="H88" s="16"/>
-      <c r="I88" s="11"/>
-      <c r="J88" s="11"/>
-      <c r="K88" s="11"/>
-      <c r="L88" s="16"/>
-      <c r="M88" s="11"/>
-      <c r="N88" s="11"/>
-      <c r="O88" s="11"/>
-      <c r="P88" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q88" s="11"/>
-      <c r="R88" s="11"/>
-      <c r="S88" s="11"/>
+      <c r="A88" s="4" t="s">
+        <v>821</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>823</v>
+      </c>
+      <c r="D88" s="7" t="s">
+        <v>824</v>
+      </c>
+      <c r="E88" s="8" t="s">
+        <v>825</v>
+      </c>
+      <c r="F88" s="8" t="s">
+        <v>826</v>
+      </c>
+      <c r="G88" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H88" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I88" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J88" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K88" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L88" s="7" t="s">
+        <v>828</v>
+      </c>
+      <c r="M88" s="8" t="s">
+        <v>829</v>
+      </c>
+      <c r="N88" s="8" t="s">
+        <v>830</v>
+      </c>
+      <c r="O88" s="8" t="s">
+        <v>831</v>
+      </c>
+      <c r="P88" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q88" s="8" t="s">
+        <v>832</v>
+      </c>
+      <c r="R88" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S88" s="8" t="s">
+        <v>833</v>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="15"/>
-      <c r="B89" s="16"/>
-      <c r="C89" s="16"/>
-      <c r="D89" s="16"/>
-      <c r="E89" s="11"/>
-      <c r="F89" s="11"/>
-      <c r="G89" s="16"/>
-      <c r="H89" s="16"/>
-      <c r="I89" s="11"/>
-      <c r="J89" s="11"/>
-      <c r="K89" s="11"/>
-      <c r="L89" s="16"/>
-      <c r="M89" s="11"/>
-      <c r="N89" s="11"/>
-      <c r="O89" s="11"/>
-      <c r="P89" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q89" s="11"/>
-      <c r="R89" s="11"/>
-      <c r="S89" s="11"/>
+      <c r="A89" s="4" t="s">
+        <v>834</v>
+      </c>
+      <c r="B89" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>835</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>836</v>
+      </c>
+      <c r="E89" s="8" t="s">
+        <v>837</v>
+      </c>
+      <c r="F89" s="8" t="s">
+        <v>826</v>
+      </c>
+      <c r="G89" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H89" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I89" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J89" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K89" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L89" s="7" t="s">
+        <v>838</v>
+      </c>
+      <c r="M89" s="8" t="s">
+        <v>839</v>
+      </c>
+      <c r="N89" s="8" t="s">
+        <v>840</v>
+      </c>
+      <c r="O89" s="8" t="s">
+        <v>841</v>
+      </c>
+      <c r="P89" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q89" s="8" t="s">
+        <v>842</v>
+      </c>
+      <c r="R89" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S89" s="8" t="s">
+        <v>843</v>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="15"/>
-      <c r="B90" s="16"/>
-      <c r="C90" s="16"/>
-      <c r="D90" s="16"/>
-      <c r="E90" s="11"/>
-      <c r="F90" s="11"/>
-      <c r="G90" s="16"/>
-      <c r="H90" s="16"/>
-      <c r="I90" s="11"/>
-      <c r="J90" s="11"/>
-      <c r="K90" s="11"/>
-      <c r="L90" s="16"/>
-      <c r="M90" s="11"/>
-      <c r="N90" s="11"/>
-      <c r="O90" s="11"/>
-      <c r="P90" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q90" s="11"/>
-      <c r="R90" s="11"/>
-      <c r="S90" s="11"/>
+      <c r="A90" s="4" t="s">
+        <v>844</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="C90" s="7" t="s">
+        <v>845</v>
+      </c>
+      <c r="D90" s="7" t="s">
+        <v>846</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>847</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>826</v>
+      </c>
+      <c r="G90" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H90" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I90" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J90" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K90" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L90" s="7" t="s">
+        <v>838</v>
+      </c>
+      <c r="M90" s="8" t="s">
+        <v>848</v>
+      </c>
+      <c r="N90" s="8" t="s">
+        <v>849</v>
+      </c>
+      <c r="O90" s="8" t="s">
+        <v>850</v>
+      </c>
+      <c r="P90" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q90" s="8" t="s">
+        <v>842</v>
+      </c>
+      <c r="R90" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S90" s="8" t="s">
+        <v>851</v>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="15"/>
-      <c r="B91" s="16"/>
-      <c r="C91" s="16"/>
-      <c r="D91" s="16"/>
-      <c r="E91" s="11"/>
-      <c r="F91" s="11"/>
-      <c r="G91" s="16"/>
-      <c r="H91" s="16"/>
-      <c r="I91" s="11"/>
-      <c r="J91" s="11"/>
-      <c r="K91" s="11"/>
-      <c r="L91" s="16"/>
-      <c r="M91" s="11"/>
-      <c r="N91" s="11"/>
-      <c r="O91" s="11"/>
-      <c r="P91" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q91" s="11"/>
-      <c r="R91" s="11"/>
-      <c r="S91" s="11"/>
+      <c r="A91" s="4" t="s">
+        <v>852</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="C91" s="7" t="s">
+        <v>854</v>
+      </c>
+      <c r="D91" s="7" t="s">
+        <v>855</v>
+      </c>
+      <c r="E91" s="8" t="s">
+        <v>856</v>
+      </c>
+      <c r="F91" s="8" t="s">
+        <v>826</v>
+      </c>
+      <c r="G91" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H91" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I91" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J91" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K91" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L91" s="7" t="s">
+        <v>857</v>
+      </c>
+      <c r="M91" s="8" t="s">
+        <v>858</v>
+      </c>
+      <c r="N91" s="8" t="s">
+        <v>859</v>
+      </c>
+      <c r="O91" s="8" t="s">
+        <v>860</v>
+      </c>
+      <c r="P91" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q91" s="8" t="s">
+        <v>861</v>
+      </c>
+      <c r="R91" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S91" s="8" t="s">
+        <v>862</v>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="15"/>
-      <c r="B92" s="16"/>
-      <c r="C92" s="16"/>
-      <c r="D92" s="16"/>
-      <c r="E92" s="11"/>
-      <c r="F92" s="11"/>
-      <c r="G92" s="16"/>
-      <c r="H92" s="16"/>
-      <c r="I92" s="11"/>
-      <c r="J92" s="11"/>
-      <c r="K92" s="11"/>
-      <c r="L92" s="16"/>
-      <c r="M92" s="11"/>
-      <c r="N92" s="11"/>
-      <c r="O92" s="11"/>
-      <c r="P92" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q92" s="11"/>
-      <c r="R92" s="11"/>
-      <c r="S92" s="11"/>
+      <c r="A92" s="4" t="s">
+        <v>863</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="C92" s="7" t="s">
+        <v>864</v>
+      </c>
+      <c r="D92" s="7" t="s">
+        <v>865</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>866</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>826</v>
+      </c>
+      <c r="G92" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H92" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I92" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J92" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K92" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L92" s="7" t="s">
+        <v>867</v>
+      </c>
+      <c r="M92" s="8" t="s">
+        <v>868</v>
+      </c>
+      <c r="N92" s="8" t="s">
+        <v>869</v>
+      </c>
+      <c r="O92" s="8" t="s">
+        <v>870</v>
+      </c>
+      <c r="P92" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q92" s="8" t="s">
+        <v>871</v>
+      </c>
+      <c r="R92" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S92" s="8" t="s">
+        <v>872</v>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="15"/>
-      <c r="B93" s="16"/>
-      <c r="C93" s="16"/>
-      <c r="D93" s="16"/>
-      <c r="E93" s="11"/>
-      <c r="F93" s="11"/>
-      <c r="G93" s="16"/>
-      <c r="H93" s="16"/>
-      <c r="I93" s="11"/>
-      <c r="J93" s="11"/>
-      <c r="K93" s="11"/>
-      <c r="L93" s="16"/>
-      <c r="M93" s="11"/>
-      <c r="N93" s="11"/>
-      <c r="O93" s="11"/>
-      <c r="P93" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q93" s="11"/>
-      <c r="R93" s="11"/>
-      <c r="S93" s="11"/>
+      <c r="A93" s="4" t="s">
+        <v>873</v>
+      </c>
+      <c r="B93" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="C93" s="7" t="s">
+        <v>874</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>875</v>
+      </c>
+      <c r="E93" s="8" t="s">
+        <v>876</v>
+      </c>
+      <c r="F93" s="8" t="s">
+        <v>877</v>
+      </c>
+      <c r="G93" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H93" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I93" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J93" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K93" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L93" s="7" t="s">
+        <v>878</v>
+      </c>
+      <c r="M93" s="8" t="s">
+        <v>879</v>
+      </c>
+      <c r="N93" s="8" t="s">
+        <v>880</v>
+      </c>
+      <c r="O93" s="8" t="s">
+        <v>881</v>
+      </c>
+      <c r="P93" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q93" s="8" t="s">
+        <v>882</v>
+      </c>
+      <c r="R93" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S93" s="8" t="s">
+        <v>883</v>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="15"/>
-      <c r="B94" s="16"/>
-      <c r="C94" s="16"/>
-      <c r="D94" s="16"/>
-      <c r="E94" s="11"/>
-      <c r="F94" s="11"/>
-      <c r="G94" s="16"/>
-      <c r="H94" s="16"/>
-      <c r="I94" s="11"/>
-      <c r="J94" s="11"/>
-      <c r="K94" s="11"/>
-      <c r="L94" s="16"/>
-      <c r="M94" s="11"/>
-      <c r="N94" s="11"/>
-      <c r="O94" s="11"/>
-      <c r="P94" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q94" s="11"/>
-      <c r="R94" s="11"/>
-      <c r="S94" s="11"/>
+      <c r="A94" s="4" t="s">
+        <v>884</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>885</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>886</v>
+      </c>
+      <c r="E94" s="8" t="s">
+        <v>887</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>826</v>
+      </c>
+      <c r="G94" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H94" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I94" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J94" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K94" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L94" s="7" t="s">
+        <v>888</v>
+      </c>
+      <c r="M94" s="8" t="s">
+        <v>889</v>
+      </c>
+      <c r="N94" s="8" t="s">
+        <v>890</v>
+      </c>
+      <c r="O94" s="8" t="s">
+        <v>891</v>
+      </c>
+      <c r="P94" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q94" s="8" t="s">
+        <v>892</v>
+      </c>
+      <c r="R94" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S94" s="8" t="s">
+        <v>893</v>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="15"/>
-      <c r="B95" s="16"/>
-      <c r="C95" s="16"/>
-      <c r="D95" s="16"/>
-      <c r="E95" s="11"/>
-      <c r="F95" s="11"/>
-      <c r="G95" s="16"/>
-      <c r="H95" s="16"/>
-      <c r="I95" s="11"/>
-      <c r="J95" s="11"/>
-      <c r="K95" s="11"/>
-      <c r="L95" s="16"/>
-      <c r="M95" s="11"/>
-      <c r="N95" s="11"/>
-      <c r="O95" s="11"/>
-      <c r="P95" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q95" s="11"/>
-      <c r="R95" s="11"/>
-      <c r="S95" s="11"/>
+      <c r="A95" s="4" t="s">
+        <v>894</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>896</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>897</v>
+      </c>
+      <c r="E95" s="8" t="s">
+        <v>898</v>
+      </c>
+      <c r="F95" s="8" t="s">
+        <v>899</v>
+      </c>
+      <c r="G95" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H95" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I95" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J95" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K95" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L95" s="7" t="s">
+        <v>900</v>
+      </c>
+      <c r="M95" s="8" t="s">
+        <v>901</v>
+      </c>
+      <c r="N95" s="8" t="s">
+        <v>902</v>
+      </c>
+      <c r="O95" s="8" t="s">
+        <v>903</v>
+      </c>
+      <c r="P95" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q95" s="8" t="s">
+        <v>904</v>
+      </c>
+      <c r="R95" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S95" s="8" t="s">
+        <v>905</v>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="15"/>
-      <c r="B96" s="16"/>
-      <c r="C96" s="16"/>
-      <c r="D96" s="16"/>
-      <c r="E96" s="11"/>
-      <c r="F96" s="11"/>
-      <c r="G96" s="16"/>
-      <c r="H96" s="16"/>
-      <c r="I96" s="11"/>
-      <c r="J96" s="11"/>
-      <c r="K96" s="11"/>
-      <c r="L96" s="16"/>
-      <c r="M96" s="11"/>
-      <c r="N96" s="11"/>
-      <c r="O96" s="11"/>
-      <c r="P96" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q96" s="11"/>
-      <c r="R96" s="11"/>
-      <c r="S96" s="11"/>
+      <c r="A96" s="4" t="s">
+        <v>906</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="C96" s="7" t="s">
+        <v>907</v>
+      </c>
+      <c r="D96" s="7" t="s">
+        <v>908</v>
+      </c>
+      <c r="E96" s="8" t="s">
+        <v>909</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>910</v>
+      </c>
+      <c r="G96" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H96" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I96" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J96" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K96" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L96" s="7" t="s">
+        <v>911</v>
+      </c>
+      <c r="M96" s="8" t="s">
+        <v>912</v>
+      </c>
+      <c r="N96" s="8" t="s">
+        <v>913</v>
+      </c>
+      <c r="O96" s="8" t="s">
+        <v>914</v>
+      </c>
+      <c r="P96" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q96" s="8" t="s">
+        <v>915</v>
+      </c>
+      <c r="R96" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S96" s="8" t="s">
+        <v>916</v>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="15"/>
-      <c r="B97" s="16"/>
-      <c r="C97" s="16"/>
-      <c r="D97" s="16"/>
-      <c r="E97" s="11"/>
-      <c r="F97" s="11"/>
-      <c r="G97" s="16"/>
-      <c r="H97" s="16"/>
-      <c r="I97" s="11"/>
-      <c r="J97" s="11"/>
-      <c r="K97" s="11"/>
-      <c r="L97" s="16"/>
-      <c r="M97" s="11"/>
-      <c r="N97" s="11"/>
-      <c r="O97" s="11"/>
-      <c r="P97" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q97" s="11"/>
-      <c r="R97" s="11"/>
-      <c r="S97" s="11"/>
+      <c r="A97" s="4" t="s">
+        <v>917</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="C97" s="7" t="s">
+        <v>918</v>
+      </c>
+      <c r="D97" s="7" t="s">
+        <v>919</v>
+      </c>
+      <c r="E97" s="8" t="s">
+        <v>920</v>
+      </c>
+      <c r="F97" s="8" t="s">
+        <v>921</v>
+      </c>
+      <c r="G97" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H97" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I97" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J97" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K97" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L97" s="7" t="s">
+        <v>922</v>
+      </c>
+      <c r="M97" s="8" t="s">
+        <v>923</v>
+      </c>
+      <c r="N97" s="8" t="s">
+        <v>924</v>
+      </c>
+      <c r="O97" s="8" t="s">
+        <v>925</v>
+      </c>
+      <c r="P97" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q97" s="8" t="s">
+        <v>926</v>
+      </c>
+      <c r="R97" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S97" s="8" t="s">
+        <v>927</v>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="15"/>
-      <c r="B98" s="16"/>
-      <c r="C98" s="16"/>
-      <c r="D98" s="16"/>
-      <c r="E98" s="11"/>
-      <c r="F98" s="11"/>
-      <c r="G98" s="16"/>
-      <c r="H98" s="16"/>
-      <c r="I98" s="11"/>
-      <c r="J98" s="11"/>
-      <c r="K98" s="11"/>
-      <c r="L98" s="16"/>
-      <c r="M98" s="11"/>
-      <c r="N98" s="11"/>
-      <c r="O98" s="11"/>
-      <c r="P98" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q98" s="11"/>
-      <c r="R98" s="11"/>
-      <c r="S98" s="11"/>
+      <c r="A98" s="4" t="s">
+        <v>928</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="C98" s="7" t="s">
+        <v>929</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>930</v>
+      </c>
+      <c r="E98" s="8" t="s">
+        <v>931</v>
+      </c>
+      <c r="F98" s="8" t="s">
+        <v>921</v>
+      </c>
+      <c r="G98" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H98" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I98" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J98" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K98" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L98" s="7" t="s">
+        <v>932</v>
+      </c>
+      <c r="M98" s="8" t="s">
+        <v>933</v>
+      </c>
+      <c r="N98" s="8" t="s">
+        <v>934</v>
+      </c>
+      <c r="O98" s="8" t="s">
+        <v>935</v>
+      </c>
+      <c r="P98" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q98" s="8" t="s">
+        <v>936</v>
+      </c>
+      <c r="R98" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S98" s="8" t="s">
+        <v>937</v>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="15"/>
-      <c r="B99" s="16"/>
-      <c r="C99" s="16"/>
-      <c r="D99" s="16"/>
-      <c r="E99" s="11"/>
-      <c r="F99" s="11"/>
-      <c r="G99" s="16"/>
-      <c r="H99" s="16"/>
-      <c r="I99" s="11"/>
-      <c r="J99" s="11"/>
-      <c r="K99" s="11"/>
-      <c r="L99" s="16"/>
-      <c r="M99" s="11"/>
-      <c r="N99" s="11"/>
-      <c r="O99" s="11"/>
-      <c r="P99" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q99" s="11"/>
-      <c r="R99" s="11"/>
-      <c r="S99" s="11"/>
+      <c r="A99" s="4" t="s">
+        <v>938</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="C99" s="7" t="s">
+        <v>939</v>
+      </c>
+      <c r="D99" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="E99" s="8" t="s">
+        <v>941</v>
+      </c>
+      <c r="F99" s="8" t="s">
+        <v>921</v>
+      </c>
+      <c r="G99" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H99" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I99" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J99" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K99" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L99" s="7" t="s">
+        <v>942</v>
+      </c>
+      <c r="M99" s="8" t="s">
+        <v>943</v>
+      </c>
+      <c r="N99" s="8" t="s">
+        <v>944</v>
+      </c>
+      <c r="O99" s="8" t="s">
+        <v>945</v>
+      </c>
+      <c r="P99" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q99" s="8" t="s">
+        <v>946</v>
+      </c>
+      <c r="R99" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S99" s="8" t="s">
+        <v>947</v>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="15"/>
-      <c r="B100" s="16"/>
-      <c r="C100" s="16"/>
-      <c r="D100" s="16"/>
-      <c r="E100" s="11"/>
-      <c r="F100" s="11"/>
-      <c r="G100" s="16"/>
-      <c r="H100" s="16"/>
-      <c r="I100" s="11"/>
-      <c r="J100" s="11"/>
-      <c r="K100" s="11"/>
-      <c r="L100" s="16"/>
-      <c r="M100" s="11"/>
-      <c r="N100" s="11"/>
-      <c r="O100" s="11"/>
-      <c r="P100" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q100" s="11"/>
-      <c r="R100" s="11"/>
-      <c r="S100" s="11"/>
+      <c r="A100" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="C100" s="7" t="s">
+        <v>949</v>
+      </c>
+      <c r="D100" s="7" t="s">
+        <v>950</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>951</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>921</v>
+      </c>
+      <c r="G100" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H100" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I100" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J100" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K100" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L100" s="7" t="s">
+        <v>867</v>
+      </c>
+      <c r="M100" s="8" t="s">
+        <v>952</v>
+      </c>
+      <c r="N100" s="8" t="s">
+        <v>953</v>
+      </c>
+      <c r="O100" s="8" t="s">
+        <v>954</v>
+      </c>
+      <c r="P100" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q100" s="8" t="s">
+        <v>955</v>
+      </c>
+      <c r="R100" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S100" s="8" t="s">
+        <v>956</v>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="15"/>
-      <c r="B101" s="16"/>
-      <c r="C101" s="16"/>
-      <c r="D101" s="16"/>
-      <c r="E101" s="11"/>
-      <c r="F101" s="11"/>
-      <c r="G101" s="16"/>
-      <c r="H101" s="16"/>
-      <c r="I101" s="11"/>
-      <c r="J101" s="11"/>
-      <c r="K101" s="11"/>
-      <c r="L101" s="16"/>
-      <c r="M101" s="11"/>
-      <c r="N101" s="11"/>
-      <c r="O101" s="11"/>
-      <c r="P101" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q101" s="11"/>
-      <c r="R101" s="11"/>
-      <c r="S101" s="11"/>
+      <c r="A101" s="4" t="s">
+        <v>957</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>958</v>
+      </c>
+      <c r="C101" s="7" t="s">
+        <v>959</v>
+      </c>
+      <c r="D101" s="7" t="s">
+        <v>960</v>
+      </c>
+      <c r="E101" s="8" t="s">
+        <v>961</v>
+      </c>
+      <c r="F101" s="8" t="s">
+        <v>921</v>
+      </c>
+      <c r="G101" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H101" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I101" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J101" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K101" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L101" s="7" t="s">
+        <v>962</v>
+      </c>
+      <c r="M101" s="8" t="s">
+        <v>963</v>
+      </c>
+      <c r="N101" s="8" t="s">
+        <v>964</v>
+      </c>
+      <c r="O101" s="8" t="s">
+        <v>965</v>
+      </c>
+      <c r="P101" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q101" s="8" t="s">
+        <v>966</v>
+      </c>
+      <c r="R101" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S101" s="8" t="s">
+        <v>967</v>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="15"/>
-      <c r="B102" s="16"/>
-      <c r="C102" s="16"/>
-      <c r="D102" s="16"/>
-      <c r="E102" s="11"/>
-      <c r="F102" s="11"/>
-      <c r="G102" s="16"/>
-      <c r="H102" s="16"/>
-      <c r="I102" s="11"/>
-      <c r="J102" s="11"/>
-      <c r="K102" s="11"/>
-      <c r="L102" s="16"/>
-      <c r="M102" s="11"/>
-      <c r="N102" s="11"/>
-      <c r="O102" s="11"/>
-      <c r="P102" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q102" s="11"/>
-      <c r="R102" s="11"/>
-      <c r="S102" s="11"/>
+      <c r="A102" s="4" t="s">
+        <v>968</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>958</v>
+      </c>
+      <c r="C102" s="7" t="s">
+        <v>969</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>970</v>
+      </c>
+      <c r="E102" s="8" t="s">
+        <v>971</v>
+      </c>
+      <c r="F102" s="8" t="s">
+        <v>921</v>
+      </c>
+      <c r="G102" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H102" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I102" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J102" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K102" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L102" s="7" t="s">
+        <v>972</v>
+      </c>
+      <c r="M102" s="8" t="s">
+        <v>973</v>
+      </c>
+      <c r="N102" s="8" t="s">
+        <v>974</v>
+      </c>
+      <c r="O102" s="8" t="s">
+        <v>975</v>
+      </c>
+      <c r="P102" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q102" s="8" t="s">
+        <v>976</v>
+      </c>
+      <c r="R102" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S102" s="8" t="s">
+        <v>977</v>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="15"/>
-      <c r="B103" s="16"/>
-      <c r="C103" s="16"/>
-      <c r="D103" s="16"/>
-      <c r="E103" s="11"/>
-      <c r="F103" s="11"/>
-      <c r="G103" s="16"/>
-      <c r="H103" s="16"/>
-      <c r="I103" s="11"/>
-      <c r="J103" s="11"/>
-      <c r="K103" s="11"/>
-      <c r="L103" s="16"/>
-      <c r="M103" s="11"/>
-      <c r="N103" s="11"/>
-      <c r="O103" s="11"/>
-      <c r="P103" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q103" s="11"/>
-      <c r="R103" s="11"/>
-      <c r="S103" s="11"/>
+      <c r="A103" s="4" t="s">
+        <v>978</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>979</v>
+      </c>
+      <c r="C103" s="7" t="s">
+        <v>980</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>981</v>
+      </c>
+      <c r="E103" s="8" t="s">
+        <v>982</v>
+      </c>
+      <c r="F103" s="8" t="s">
+        <v>983</v>
+      </c>
+      <c r="G103" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H103" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I103" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J103" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K103" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L103" s="7" t="s">
+        <v>984</v>
+      </c>
+      <c r="M103" s="8" t="s">
+        <v>985</v>
+      </c>
+      <c r="N103" s="8" t="s">
+        <v>986</v>
+      </c>
+      <c r="O103" s="8" t="s">
+        <v>987</v>
+      </c>
+      <c r="P103" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q103" s="8" t="s">
+        <v>988</v>
+      </c>
+      <c r="R103" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S103" s="8" t="s">
+        <v>989</v>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="15"/>
-      <c r="B104" s="16"/>
-      <c r="C104" s="16"/>
-      <c r="D104" s="16"/>
-      <c r="E104" s="11"/>
-      <c r="F104" s="11"/>
-      <c r="G104" s="16"/>
-      <c r="H104" s="16"/>
-      <c r="I104" s="11"/>
-      <c r="J104" s="11"/>
-      <c r="K104" s="11"/>
-      <c r="L104" s="16"/>
-      <c r="M104" s="11"/>
-      <c r="N104" s="11"/>
-      <c r="O104" s="11"/>
-      <c r="P104" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q104" s="11"/>
-      <c r="R104" s="11"/>
-      <c r="S104" s="11"/>
+      <c r="A104" s="4" t="s">
+        <v>990</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>991</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>992</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>993</v>
+      </c>
+      <c r="E104" s="8" t="s">
+        <v>994</v>
+      </c>
+      <c r="F104" s="8" t="s">
+        <v>995</v>
+      </c>
+      <c r="G104" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H104" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I104" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="J104" s="14">
+        <v>46196.0</v>
+      </c>
+      <c r="K104" s="8" t="s">
+        <v>827</v>
+      </c>
+      <c r="L104" s="7" t="s">
+        <v>996</v>
+      </c>
+      <c r="M104" s="8" t="s">
+        <v>997</v>
+      </c>
+      <c r="N104" s="8" t="s">
+        <v>998</v>
+      </c>
+      <c r="O104" s="8" t="s">
+        <v>999</v>
+      </c>
+      <c r="P104" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q104" s="8" t="s">
+        <v>1000</v>
+      </c>
+      <c r="R104" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S104" s="8" t="s">
+        <v>1001</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="15"/>
@@ -9129,27 +10512,25 @@
       <c r="S140" s="11"/>
     </row>
     <row r="141">
-      <c r="A141" s="15"/>
-      <c r="B141" s="16"/>
-      <c r="C141" s="16"/>
-      <c r="D141" s="16"/>
-      <c r="E141" s="11"/>
-      <c r="F141" s="11"/>
-      <c r="G141" s="16"/>
-      <c r="H141" s="16"/>
-      <c r="I141" s="11"/>
-      <c r="J141" s="11"/>
-      <c r="K141" s="11"/>
-      <c r="L141" s="16"/>
-      <c r="M141" s="11"/>
-      <c r="N141" s="11"/>
-      <c r="O141" s="11"/>
-      <c r="P141" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q141" s="11"/>
-      <c r="R141" s="11"/>
-      <c r="S141" s="11"/>
+      <c r="A141" s="4"/>
+      <c r="B141" s="5"/>
+      <c r="C141" s="7"/>
+      <c r="D141" s="7"/>
+      <c r="E141" s="8"/>
+      <c r="F141" s="8"/>
+      <c r="G141" s="7"/>
+      <c r="H141" s="7"/>
+      <c r="I141" s="8"/>
+      <c r="J141" s="8"/>
+      <c r="K141" s="8"/>
+      <c r="L141" s="5"/>
+      <c r="M141" s="8"/>
+      <c r="N141" s="8"/>
+      <c r="O141" s="8"/>
+      <c r="P141" s="8"/>
+      <c r="Q141" s="8"/>
+      <c r="R141" s="8"/>
+      <c r="S141" s="8"/>
     </row>
     <row r="142">
       <c r="A142" s="15"/>
@@ -9175,25 +10556,27 @@
       <c r="S142" s="11"/>
     </row>
     <row r="143">
-      <c r="A143" s="4"/>
-      <c r="B143" s="5"/>
-      <c r="C143" s="7"/>
-      <c r="D143" s="7"/>
-      <c r="E143" s="8"/>
-      <c r="F143" s="8"/>
-      <c r="G143" s="7"/>
-      <c r="H143" s="7"/>
-      <c r="I143" s="8"/>
-      <c r="J143" s="8"/>
-      <c r="K143" s="8"/>
-      <c r="L143" s="5"/>
-      <c r="M143" s="8"/>
-      <c r="N143" s="8"/>
-      <c r="O143" s="8"/>
-      <c r="P143" s="8"/>
-      <c r="Q143" s="8"/>
-      <c r="R143" s="8"/>
-      <c r="S143" s="8"/>
+      <c r="A143" s="15"/>
+      <c r="B143" s="16"/>
+      <c r="C143" s="16"/>
+      <c r="D143" s="16"/>
+      <c r="E143" s="11"/>
+      <c r="F143" s="11"/>
+      <c r="G143" s="16"/>
+      <c r="H143" s="16"/>
+      <c r="I143" s="11"/>
+      <c r="J143" s="11"/>
+      <c r="K143" s="11"/>
+      <c r="L143" s="16"/>
+      <c r="M143" s="11"/>
+      <c r="N143" s="11"/>
+      <c r="O143" s="11"/>
+      <c r="P143" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q143" s="11"/>
+      <c r="R143" s="11"/>
+      <c r="S143" s="11"/>
     </row>
     <row r="144">
       <c r="A144" s="15"/>
@@ -28538,64 +29921,18 @@
       <c r="R984" s="11"/>
       <c r="S984" s="11"/>
     </row>
-    <row r="985">
-      <c r="A985" s="15"/>
-      <c r="B985" s="16"/>
-      <c r="C985" s="16"/>
-      <c r="D985" s="16"/>
-      <c r="E985" s="11"/>
-      <c r="F985" s="11"/>
-      <c r="G985" s="16"/>
-      <c r="H985" s="16"/>
-      <c r="I985" s="11"/>
-      <c r="J985" s="11"/>
-      <c r="K985" s="11"/>
-      <c r="L985" s="16"/>
-      <c r="M985" s="11"/>
-      <c r="N985" s="11"/>
-      <c r="O985" s="11"/>
-      <c r="P985" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q985" s="11"/>
-      <c r="R985" s="11"/>
-      <c r="S985" s="11"/>
-    </row>
-    <row r="986">
-      <c r="A986" s="15"/>
-      <c r="B986" s="16"/>
-      <c r="C986" s="16"/>
-      <c r="D986" s="16"/>
-      <c r="E986" s="11"/>
-      <c r="F986" s="11"/>
-      <c r="G986" s="16"/>
-      <c r="H986" s="16"/>
-      <c r="I986" s="11"/>
-      <c r="J986" s="11"/>
-      <c r="K986" s="11"/>
-      <c r="L986" s="16"/>
-      <c r="M986" s="11"/>
-      <c r="N986" s="11"/>
-      <c r="O986" s="11"/>
-      <c r="P986" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q986" s="11"/>
-      <c r="R986" s="11"/>
-      <c r="S986" s="11"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B986">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B984">
       <formula1>"Rules,Trades,Resolution,Communication,Other,News,Wallets,Blockchain,Trades"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="R2:R986">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="R2:R984">
       <formula1>"Public,Claimant-Private,Counsel-Only,Attorney review,Internal,Restricted"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N2:N986">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N2:N984">
       <formula1>"Verified,Partially Verified,Unverified,Derived analysis"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:J986">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:J984">
       <formula1>OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D"))</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
more evidence and standarized evidence folder
</commit_message>
<xml_diff>
--- a/Evidence Register.xlsx
+++ b/Evidence Register.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1687" uniqueCount="1002">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2231" uniqueCount="1331">
   <si>
     <t>Evidence ID</t>
   </si>
@@ -3137,6 +3137,1125 @@
   </si>
   <si>
     <t>Use as an orientation note only. The underlying CSVs and transaction hashes remain the primary evidence.</t>
+  </si>
+  <si>
+    <t>DCE-002</t>
+  </si>
+  <si>
+    <t>01_Originals/UMA_1775946625_Thread _1492668186179666113/UMA - 💬｜dispute-threads - Will _Donk_ be said during the PGL Bucharest 2026 Grand Final_ - 1775946625 [1492668186179666113].html</t>
+  </si>
+  <si>
+    <t>DCE-002_UMA_Donk_thread_original.html</t>
+  </si>
+  <si>
+    <t>Authenticated HTML export of the UMA dispute thread for the Donk market, including the full captured thread context.</t>
+  </si>
+  <si>
+    <t>UMA Discord export</t>
+  </si>
+  <si>
+    <t>Omer/SatlaMocha</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/718590743446290492/1492668186179666113</t>
+  </si>
+  <si>
+    <t>Prior UMA dispute thread / voter coordination context</t>
+  </si>
+  <si>
+    <t>Preserves the readable thread context for prior UMA dispute discussion and screenshots involving disputed voting positions, whale/token influence language, and market-resolution conduct.</t>
+  </si>
+  <si>
+    <t>DCE-003; DCE-010; DCE-017; DCE-020</t>
+  </si>
+  <si>
+    <t>ce4e941ea499c098714f5022bf341796d4d81992b7d0d4b53c5119d63f4a2422</t>
+  </si>
+  <si>
+    <t>File integrity verified by SHA-256. Export is preserved in Discord Exports package.</t>
+  </si>
+  <si>
+    <t>DCE-003</t>
+  </si>
+  <si>
+    <t>01_Originals/UMA_1775946625_Thread _1492668186179666113/UMA - 💬｜dispute-threads - Will _Donk_ be said during the PGL Bucharest 2026 Grand Final_ - 1775946625 [1492668186179666113].json</t>
+  </si>
+  <si>
+    <t>DCE-003_UMA_Donk_thread_original.json</t>
+  </si>
+  <si>
+    <t>Authenticated JSON export of the UMA dispute thread for the Donk market, including message IDs, authors, timestamps, reactions, embeds, and message content.</t>
+  </si>
+  <si>
+    <t>Machine-readable source export that supports authentication of the Donk thread screenshots and allows counsel to inspect message IDs, author IDs, timestamps, and full context.</t>
+  </si>
+  <si>
+    <t>DCE-002; DCE-010; DCE-017; DCE-020</t>
+  </si>
+  <si>
+    <t>d70275b64d09bf505642e40eddb751496133eee12234328278c9882d4e972ffb</t>
+  </si>
+  <si>
+    <t>DCE-004</t>
+  </si>
+  <si>
+    <t>01_Originals/UMA_Channel_719352532354465833/UMA _719352532354465833_03_07_2025_to_06_07_2025.html</t>
+  </si>
+  <si>
+    <t>DCE-004_UMA_voting_discussion_2025-07-03_to_2025-07-06_original.html</t>
+  </si>
+  <si>
+    <t>Authenticated HTML export of the UMA voting-discussion channel for the captured July 2025 window.</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/718590743446290492/719352532354465833</t>
+  </si>
+  <si>
+    <t>UMA voting discussion / coordination evidence</t>
+  </si>
+  <si>
+    <t>Preserves the readable channel context for borntoolate-related messages and surrounding discussion, including vote-reveal timing, whale consultation, united-front language, and agreement-performance language.</t>
+  </si>
+  <si>
+    <t>DCE-005; DCE-008; DCE-011; DCE-014; DCE-015; DCE-017; DCE-020</t>
+  </si>
+  <si>
+    <t>cb1474253dcf1b2a5768502c5f2a625348c84828caca2a1717be5dd6726d145c</t>
+  </si>
+  <si>
+    <t>DCE-005</t>
+  </si>
+  <si>
+    <t>01_Originals/UMA_Channel_719352532354465833/UMA _719352532354465833_03_07_2025_to_06_07_2025.json</t>
+  </si>
+  <si>
+    <t>DCE-005_UMA_voting_discussion_2025-07-03_to_2025-07-06_original.json</t>
+  </si>
+  <si>
+    <t>Authenticated JSON export of the UMA voting-discussion channel for the captured July 2025 window.</t>
+  </si>
+  <si>
+    <t>Machine-readable source export proving message IDs, author IDs, timestamps, and full context for borntoolate-related coordination messages and related screenshot evidence.</t>
+  </si>
+  <si>
+    <t>DCE-004; DCE-008; DCE-011; DCE-014; DCE-015; DCE-017; DCE-020</t>
+  </si>
+  <si>
+    <t>83548a8c3e32727088d56be416202d85536eaf9f858e38409867851824b99fa0</t>
+  </si>
+  <si>
+    <t>DCE-006</t>
+  </si>
+  <si>
+    <t>01_Originals/UMA_Thread_1515853475681009704/UMA - 💬｜dispute-threads - US x Iran permanent peace deal by June 15, 2026_ - 1781475979 [1515853475681009704].html</t>
+  </si>
+  <si>
+    <t>DCE-006_UMA_US_Iran_June15_thread_original.html</t>
+  </si>
+  <si>
+    <t>Authenticated HTML export of the UMA dispute thread for the US x Iran permanent peace deal by June 15, 2026 market.</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/718590743446290492/1515853475681009704</t>
+  </si>
+  <si>
+    <t>US x Iran market dispute / UMA resolution discussion</t>
+  </si>
+  <si>
+    <t>Preserves readable thread context showing arguments about whether the market was too early, whether the agreement was interim or permanent, and contemporaneous discussion before or during the disputed resolution process.</t>
+  </si>
+  <si>
+    <t>DCE-007; DCE-009; DCE-016; DCE-017; DCE-020</t>
+  </si>
+  <si>
+    <t>e8944a8dfea612f7551350a20633cca2fb4e69f535dc7e886f52c7a962b82d0f</t>
+  </si>
+  <si>
+    <t>DCE-007</t>
+  </si>
+  <si>
+    <t>01_Originals/UMA_Thread_1515853475681009704/UMA - 💬｜dispute-threads - US x Iran permanent peace deal by June 15, 2026_ - 1781475979 [1515853475681009704].json</t>
+  </si>
+  <si>
+    <t>DCE-007_UMA_US_Iran_June15_thread_original.json</t>
+  </si>
+  <si>
+    <t>Authenticated JSON export of the UMA dispute thread for the US x Iran permanent peace deal by June 15, 2026 market.</t>
+  </si>
+  <si>
+    <t>Machine-readable source export that supports authentication of US x Iran thread messages, author IDs, timestamps, message IDs, and the context for drespasmo/Lazarus screenshots.</t>
+  </si>
+  <si>
+    <t>DCE-006; DCE-009; DCE-016; DCE-017; DCE-020</t>
+  </si>
+  <si>
+    <t>acf69026d4443d129995c58a18cba0a8cb6d3cbdb5d3174c0a4fdabb6efb3e00</t>
+  </si>
+  <si>
+    <t>DCE-008</t>
+  </si>
+  <si>
+    <t>02_Readable_HTML/UMA _719352532354465833_03_07_2025_to_06_07_2025.html</t>
+  </si>
+  <si>
+    <t>DCE-008_UMA_voting_discussion_2025-07-03_to_2025-07-06_readable.html</t>
+  </si>
+  <si>
+    <t>Readable HTML copy of the UMA voting-discussion channel export for counsel review.</t>
+  </si>
+  <si>
+    <t>Counsel-friendly readable copy of the authenticated channel export that contains borntoolate-related message context.</t>
+  </si>
+  <si>
+    <t>DCE-004; DCE-005; DCE-011; DCE-014; DCE-015; DCE-017; DCE-020</t>
+  </si>
+  <si>
+    <t>DCE-009</t>
+  </si>
+  <si>
+    <t>02_Readable_HTML/UMA_1781475979_1515853475681009704.html</t>
+  </si>
+  <si>
+    <t>DCE-009_UMA_US_Iran_June15_thread_readable.html</t>
+  </si>
+  <si>
+    <t>Readable HTML copy of the UMA US x Iran permanent peace deal thread export for counsel review.</t>
+  </si>
+  <si>
+    <t>Counsel-friendly readable copy of the authenticated US x Iran thread export.</t>
+  </si>
+  <si>
+    <t>DCE-006; DCE-007; DCE-016; DCE-017; DCE-020</t>
+  </si>
+  <si>
+    <t>DCE-010</t>
+  </si>
+  <si>
+    <t>03_Screenshot_Context/HLpHylzagAAbWDx.png</t>
+  </si>
+  <si>
+    <t>DCE-010_Davy_Jones_UMA_tokens_force_it_through.png</t>
+  </si>
+  <si>
+    <t>Preserved screenshot showing a UMA-tagged account appearing to state “P1 - No,” “We have more UMA tokens,” and “Force it through.”</t>
+  </si>
+  <si>
+    <t>Screenshot context preserved in Discord export package</t>
+  </si>
+  <si>
+    <t>unknown</t>
+  </si>
+  <si>
+    <t>UMA token influence / vote coordination screenshot</t>
+  </si>
+  <si>
+    <t>Relevant to process-integrity and vote-influence issues because it captures language about the correct outcome, UMA token power, investment protection, and forcing an outcome.</t>
+  </si>
+  <si>
+    <t>DCE-001; DCE-017; DCE-018</t>
+  </si>
+  <si>
+    <t>45e588852ee0c087069eaa5dcc1d468d44d9625792f3648703cf97a42a54d344</t>
+  </si>
+  <si>
+    <t>Screenshot file is preserved and hashed. Underlying message link was not identified from the exports in this package. File integrity verified by SHA-256.</t>
+  </si>
+  <si>
+    <t>DCE-011</t>
+  </si>
+  <si>
+    <t>03_Screenshot_Context/HLpICwha8AEY4tZ.png</t>
+  </si>
+  <si>
+    <t>DCE-011_borntoolate_other_whales_same_page.png</t>
+  </si>
+  <si>
+    <t>Preserved screenshot showing borntoolate/lifewillbeokay message: “I will consult with the other whales to make sure we’re all on the same page,” followed by “Showing a united front is critical for this vote.”</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/718590743446290492/719352532354465833/1390809434531303494</t>
+  </si>
+  <si>
+    <t>Authenticated screenshot and export-supported message evidence relevant to whale coordination language, vote alignment, and UMA voting-process integrity.</t>
+  </si>
+  <si>
+    <t>DCE-004; DCE-005; DCE-008; DCE-017; DCE-018; DCE-020</t>
+  </si>
+  <si>
+    <t>917440dc050211ea21abba9d03938c580aeb53797976b9ca75c42f303d83eb11</t>
+  </si>
+  <si>
+    <t>Message metadata is also indexed in UMA whale messages.xlsx and supported by the JSON/HTML channel export.</t>
+  </si>
+  <si>
+    <t>DCE-012</t>
+  </si>
+  <si>
+    <t>03_Screenshot_Context/image.png</t>
+  </si>
+  <si>
+    <t>DCE-012_public_commentary_yes_whales_interim_mou.png</t>
+  </si>
+  <si>
+    <t>Preserved screenshot of public commentary alleging YES whales relied on an interim temporary MoU interpretation in the US/Iran permanent peace deal context.</t>
+  </si>
+  <si>
+    <t>US x Iran market public commentary / context</t>
+  </si>
+  <si>
+    <t>Supports context for the claimant theory that the YES outcome relied on an interim or temporary MoU interpretation rather than the permanent peace deal criteria.</t>
+  </si>
+  <si>
+    <t>DCE-001; DCE-018</t>
+  </si>
+  <si>
+    <t>6aa83497028adb5e501143af6eda1083cfabf596941840128b3b13f7388a6aea</t>
+  </si>
+  <si>
+    <t>Supporting context screenshot. Treat as contextual evidence rather than primary source proof of the market criteria. File integrity verified by SHA-256.</t>
+  </si>
+  <si>
+    <t>DCE-013</t>
+  </si>
+  <si>
+    <t>03_Screenshot_Context/Screenshot 2026-06-25 225656.png</t>
+  </si>
+  <si>
+    <t>DCE-013_Verdit_X_post_UMA_token_holder_warning.png</t>
+  </si>
+  <si>
+    <t>Preserved screenshot of a public X/Twitter post warning about Polymarket and referencing Discord chat records involving a large UMA token holder discussing market resolution.</t>
+  </si>
+  <si>
+    <t>Public dissemination of UMA coordination evidence</t>
+  </si>
+  <si>
+    <t>Shows public reporting/dissemination context for the Discord coordination screenshots and process-integrity concerns.</t>
+  </si>
+  <si>
+    <t>DCE-010; DCE-011; DCE-018</t>
+  </si>
+  <si>
+    <t>7eb27b1bdf0d3d8a7392d73c631602b1c44ff7dabecb3fc321a07f1b52c0ee03</t>
+  </si>
+  <si>
+    <t>Source URL was not included in the archive. File integrity verified by SHA-256.</t>
+  </si>
+  <si>
+    <t>DCE-014</t>
+  </si>
+  <si>
+    <t>03_Screenshot_Context/Screenshot 2026-06-25 230359.png</t>
+  </si>
+  <si>
+    <t>DCE-014_borntoolate_message_context_search_result.png</t>
+  </si>
+  <si>
+    <t>Preserved screenshot of UMA voting-discussion context showing the borntoolate/lifewillbeokay “other whales” message in Discord search/context view.</t>
+  </si>
+  <si>
+    <t>Supports authentication and context for the borntoolate whale-consultation message through visible Discord UI context and matching JSON/HTML export records.</t>
+  </si>
+  <si>
+    <t>DCE-004; DCE-005; DCE-008; DCE-011; DCE-017; DCE-018; DCE-020</t>
+  </si>
+  <si>
+    <t>335b9d49426d59da5a543dcd2453f560ea268e53caebcfe65702939251bbe14a</t>
+  </si>
+  <si>
+    <t>Screenshot capture date appears in filename. Message date is 2025-07-04 UTC.</t>
+  </si>
+  <si>
+    <t>DCE-015</t>
+  </si>
+  <si>
+    <t>03_Screenshot_Context/Screenshot 2026-06-26 114208.png</t>
+  </si>
+  <si>
+    <t>DCE-015_borntoolate_fulfilled_my_part_agreement.png</t>
+  </si>
+  <si>
+    <t>Preserved screenshot showing borntoolate/lifewillbeokay message: “I fulfilled my part of the agreement. Now you must fulfill yours.”</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/718590743446290492/719352532354465833/1390829921844068493</t>
+  </si>
+  <si>
+    <t>Authenticated screenshot and export-supported message evidence relevant to agreement-performance language in the same voting-discussion context.</t>
+  </si>
+  <si>
+    <t>DCE-004; DCE-005; DCE-008; DCE-011; DCE-014; DCE-017; DCE-018; DCE-020</t>
+  </si>
+  <si>
+    <t>388a2ef8240031efb4f5a26e033a669bf41e425f0218f1311e5fa428640808a7</t>
+  </si>
+  <si>
+    <t>Message metadata is also indexed in UMA whale messages.xlsx and supported by JSON/HTML channel export.</t>
+  </si>
+  <si>
+    <t>DCE-016</t>
+  </si>
+  <si>
+    <t>03_Screenshot_Context/Screenshot 2026-06-26 114557.png</t>
+  </si>
+  <si>
+    <t>DCE-016_drespasmo_Lazarus_US_Iran_dispute_context.png</t>
+  </si>
+  <si>
+    <t>Preserved screenshot from the US x Iran dispute thread showing messages about the market being too early / interim MoU, plus a drespasmo/Lazarus message stating “P2 - YES Because corruption is only bad if I’m not involved.”</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/718590743446290492/1515853475681009704/1515983186696339568</t>
+  </si>
+  <si>
+    <t>Authenticated screenshot and export-supported message evidence relevant to the US x Iran thread, including contemporaneous dispute arguments and a preserved statement by drespasmo/Lazarus.</t>
+  </si>
+  <si>
+    <t>DCE-006; DCE-007; DCE-009; DCE-017; DCE-018; DCE-020</t>
+  </si>
+  <si>
+    <t>e83ba9e8a9383ce1332aa4de561e7853e6b437b2061a243d8905aa16c1115a86</t>
+  </si>
+  <si>
+    <t>Message metadata is also indexed in UMA whale messages.xlsx and supported by the JSON/HTML thread export.</t>
+  </si>
+  <si>
+    <t>DCE-017</t>
+  </si>
+  <si>
+    <t>03_Screenshot_Context/Screenshot_2026-06-25-21-32-00-92_572064f74bd5f9fa804b05334aa4f912.jpg</t>
+  </si>
+  <si>
+    <t>DCE-017_Donk_thread_vote_argument_largest_NO_holder.png</t>
+  </si>
+  <si>
+    <t>Preserved mobile screenshot of the Donk dispute thread showing a P2 argument about the largest NO holder allegedly hearing “donk” and voting/trading incentives.</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/718590743446290492/1492668186179666113/1494099459557032027</t>
+  </si>
+  <si>
+    <t>Relevant as prior dispute-thread context involving allegations about voting incentives, market positions, and outcome arguments in UMA-related dispute discussion.</t>
+  </si>
+  <si>
+    <t>DCE-002; DCE-003; DCE-010; DCE-018</t>
+  </si>
+  <si>
+    <t>9526da52380baf62167410bdbcf9442d19f43c8f7b4a7e5516607062138dc869</t>
+  </si>
+  <si>
+    <t>Actual zip-contained image hash differs from the Images_original_hashes_sha256.csv entry for the similarly named uploaded file. SHA-256 in this row is computed from the file inside Discord Exports.zip.</t>
+  </si>
+  <si>
+    <t>DCE-018</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>05_Hashes/Discord_Exports_hashes_sha256_manifest.csv</t>
+  </si>
+  <si>
+    <t>DCE-018_Discord_exports_SHA256_manifest.csv</t>
+  </si>
+  <si>
+    <t>SHA-256, SHA-1, and MD5 manifest for the Discord JSON/HTML export files.</t>
+  </si>
+  <si>
+    <t>Local hash manifest in Discord Exports/05_Hashes</t>
+  </si>
+  <si>
+    <t>Evidence integrity / hash preservation</t>
+  </si>
+  <si>
+    <t>Provides file integrity records for the original Discord JSON/HTML exports and supports authentication of the exported records.</t>
+  </si>
+  <si>
+    <t>DCE-002; DCE-003; DCE-004; DCE-005; DCE-006; DCE-007; DCE-008; DCE-009</t>
+  </si>
+  <si>
+    <t>979c8536684c9f08b722f05ebe4410d2ace3a9a963f9e30edb18fa1b30a7bfc0</t>
+  </si>
+  <si>
+    <t>Manifest includes hashed_at_utc values. SHA-256 in this row is the hash of the manifest file itself.</t>
+  </si>
+  <si>
+    <t>DCE-019</t>
+  </si>
+  <si>
+    <t>05_Hashes/Images_original_hashes_sha256.csv</t>
+  </si>
+  <si>
+    <t>DCE-019_Discord_screenshot_images_SHA256_manifest.csv</t>
+  </si>
+  <si>
+    <t>SHA-256 manifest for screenshot context image files included in the Discord export package.</t>
+  </si>
+  <si>
+    <t>Provides file integrity records for screenshot context files, including borntoolate-related and US x Iran dispute screenshots.</t>
+  </si>
+  <si>
+    <t>DCE-010; DCE-011; DCE-012; DCE-013; DCE-014; DCE-015; DCE-016; DCE-017</t>
+  </si>
+  <si>
+    <t>c5fc423c837e8cf3f1777c9984db1fdd6d77b73cfb671b4cce4205a699719897</t>
+  </si>
+  <si>
+    <t>Manifest is preserved and hashed. One screenshot filename has a zip-contained file hash that differs from the original image manifest entry; use the actual file hash from the row when preserving the zip-contained copy.</t>
+  </si>
+  <si>
+    <t>DCE-020</t>
+  </si>
+  <si>
+    <t>UMA whale messages.xlsx</t>
+  </si>
+  <si>
+    <t>DCE-020_UMA_whale_messages_index.xlsx</t>
+  </si>
+  <si>
+    <t>Compiled index of selected UMA whale / coordination messages, including username, author ID, message ID, channel/thread ID, server ID, original message link, timestamp, screenshot filename, and screenshot hash.</t>
+  </si>
+  <si>
+    <t>Derived index prepared from Discord exports and screenshot hash records</t>
+  </si>
+  <si>
+    <t>UMA voting discussion / coordination evidence index</t>
+  </si>
+  <si>
+    <t>Counsel-facing index tying selected borntoolate and drespasmo/Lazarus screenshots to Discord message IDs, author IDs, timestamps, direct message links, and screenshot hashes.</t>
+  </si>
+  <si>
+    <t>DCE-011; DCE-014; DCE-015; DCE-016; DCE-018; DCE-019</t>
+  </si>
+  <si>
+    <t>8e04674dd78483f5a9cdb36ad910d1ced075f863a87ff5e15144da2b8da86697</t>
+  </si>
+  <si>
+    <t>This is a derived index, not the primary source. Primary source support is the JSON/HTML export files, screenshot files, and hash manifests.</t>
+  </si>
+  <si>
+    <t>EVC-001</t>
+  </si>
+  <si>
+    <t>POLYMARKET UMA scam - 🔍 ┃ EVIDENCE &amp; RESEARCH - 📂┃evidences [1517091731236192418].json</t>
+  </si>
+  <si>
+    <t>Discord Exports/EVC-001_evidence_channel_export.html</t>
+  </si>
+  <si>
+    <t>Authenticated export of the POLYMARKET UMA scam evidence channel used as provenance for submitted evidence, screenshots, source links, and attachments. The uploaded file has .json extension but contains an HTML Discord export.</t>
+  </si>
+  <si>
+    <t>Discord channel export</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418</t>
+  </si>
+  <si>
+    <t>Discord export timestamp; market deadline should be reviewed in ET; blockchain records should be reviewed in UTC</t>
+  </si>
+  <si>
+    <t>Evidence collection / Discord provenance</t>
+  </si>
+  <si>
+    <t>Preserves message IDs, submitters, timestamps, context, and source links for evidence submitted in the evidence channel.</t>
+  </si>
+  <si>
+    <t>DCE-018; DCE-019</t>
+  </si>
+  <si>
+    <t>Discord Exports/EVC-001_evidence_channel_export.html: 1b2d4118b8c4ca8c408a5bc3746bab3d51b49e09824102ad43f121762f7ef523</t>
+  </si>
+  <si>
+    <t>Only the export file is included here. Font, style, script, and avatar assets from the export package were not copied into the organized evidence folder.</t>
+  </si>
+  <si>
+    <t>EVC-002</t>
+  </si>
+  <si>
+    <t>News</t>
+  </si>
+  <si>
+    <t>Assets/image-c32eff51cca1851e.png</t>
+  </si>
+  <si>
+    <t>News and Goverment Sources/EVC-002_01_image-c32eff51cca1851e.png</t>
+  </si>
+  <si>
+    <t>Submitted news/video screenshot showing President Trump speaking at the G7 context with a caption indicating the United States would most likely sign a deal with Iran.</t>
+  </si>
+  <si>
+    <t>Discord evidence channel export and preserved attachment assets</t>
+  </si>
+  <si>
+    <t>Gujii</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517092453675565130</t>
+  </si>
+  <si>
+    <t>Rule condition / public-source timeline</t>
+  </si>
+  <si>
+    <t>Supports the timeline and the distinction between an expected future signing and an agreement already qualifying by the June 15 deadline.</t>
+  </si>
+  <si>
+    <t>EV-01; RULE-NO-001; RULE-NO-004</t>
+  </si>
+  <si>
+    <t>News and Goverment Sources/EVC-002_01_image-c32eff51cca1851e.png: caedfca73fbb749e8aff6942b1add526dcf50e7253b8349e63de58378ba0655e</t>
+  </si>
+  <si>
+    <t>Content should be checked against the original video/source. File preservation and hash are verified.</t>
+  </si>
+  <si>
+    <t>EVC-003</t>
+  </si>
+  <si>
+    <t>Assets/0D1231DD-F7F6-4549-AC4D-E4F50B0CBED2-4fba38ca36279654.png
+Assets/Screenshot_2026-06-18-12-58-45-16_f052540a-61d5f47e849f384e.jpg</t>
+  </si>
+  <si>
+    <t>Market Rules/EVC-003_01_0D1231DD-F7F6-4549-AC4D-E4F50B0CBED2-4fba38ca36279654.png
+Market Rules/EVC-003_02_Screenshot_2026-06-18-12-58-45-16_f052540a-61d5f47e849f384e.jpg</t>
+  </si>
+  <si>
+    <t>Additional mobile screenshots of the June 15 market rule text, claimant position context, dispute steps, and final YES outcome display.</t>
+  </si>
+  <si>
+    <t>Teh Golden Buddha / unknown forwarded submitter</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517114934419390606
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517115048848396398</t>
+  </si>
+  <si>
+    <t>Market rules / final resolution / claimant position</t>
+  </si>
+  <si>
+    <t>Corroborates the written market criteria, the NO position context, the repeated dispute path, and the final YES outcome shown to users.</t>
+  </si>
+  <si>
+    <t>PM-RULE-001; PM-RULE-002; PM-RES-001; PM-RULE-003</t>
+  </si>
+  <si>
+    <t>Market Rules/EVC-003_01_0D1231DD-F7F6-4549-AC4D-E4F50B0CBED2-4fba38ca36279654.png: 1db63337e749e0f0c9749a04c9a46aa90775c74188b823605a89680e080e58e8
+Market Rules/EVC-003_02_Screenshot_2026-06-18-12-58-45-16_f052540a-61d5f47e849f384e.jpg: fc6c72a6f32ac09e830080ab03614e30082dcb3ac8f5813f2ff96cfa29da00fe</t>
+  </si>
+  <si>
+    <t>Includes additional captures not already represented by the existing PM-RULE and PM-RES rows. Treat as corroborating screenshots, not independent legal conclusions.</t>
+  </si>
+  <si>
+    <t>EVC-004</t>
+  </si>
+  <si>
+    <t>Assets/image-eacb0676c2672ae6.png
+Assets/image-7cada7c433778219.png
+Assets/image-6529976488f15551.png
+Assets/image-495bdba35fd6ddc9.png</t>
+  </si>
+  <si>
+    <t>News and Goverment Sources/EVC-004_01_image-eacb0676c2672ae6.png
+News and Goverment Sources/EVC-004_03_image-7cada7c433778219.png
+News and Goverment Sources/EVC-004_04_image-6529976488f15551.png
+News and Goverment Sources/EVC-004_05_image-495bdba35fd6ddc9.png</t>
+  </si>
+  <si>
+    <t>Screenshots submitted as rebuttal material concerning electronic signing, Bloomberg’s draft memorandum coverage, and whether the alleged document satisfied the market rule requirement.</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517124610804547614
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517124935590477875</t>
+  </si>
+  <si>
+    <t>Rule condition / Bloomberg draft / signature dispute</t>
+  </si>
+  <si>
+    <t>Supports the claimant theory that alleged electronic or draft materials did not satisfy the written rule requiring a qualifying permanent peace agreement by the deadline.</t>
+  </si>
+  <si>
+    <t>EV-02; EV-04; RULE-NO-005; RULE-NO-006; RULE-NO-007</t>
+  </si>
+  <si>
+    <t>News and Goverment Sources/EVC-004_01_image-eacb0676c2672ae6.png: ad6779abda2a1213f476f176a27f23c922a0295c8d37a366a23a4cbeeb0d4fbd
+News and Goverment Sources/EVC-004_03_image-7cada7c433778219.png: c27a7dee8a0e716e3a1676bee8c6588309f155ad03d3d6b2f540a7d94c6d89f7
+News and Goverment Sources/EVC-004_04_image-6529976488f15551.png: fee9ccbb0d44126680706b476b806c41eb85b3e10f253d060db345bd7c7e4260
+News and Goverment Sources/EVC-004_05_image-495bdba35fd6ddc9.png: 083f1c9a17768abb41ad5b158ed7bba2f05976bc4c6e410db6af77dd7939bc39</t>
+  </si>
+  <si>
+    <t>Screenshots preserve submitted source material and arguments. Counsel should verify the underlying articles and rule text independently. Duplicate file image-1df6cfa86ff16f36.png was not included because its SHA-256 hash was already present in the existing register.</t>
+  </si>
+  <si>
+    <t>EVC-005</t>
+  </si>
+  <si>
+    <t>Assets/IMG_2121-7b6e3c30fde93c7c.png
+Assets/IMG_2122-8e3e775c9143519c.png
+Assets/IMG_2123-ff4e4bcfd71229ac.png
+Assets/IMG_3526-7bd2193fb2ae45ba.jpg
+Assets/IMG_3524-8eaf21a3cadadac4.jpg
+Assets/IMG_3482-ca26986df53d8d39.png
+Assets/message-22503970b78b530b.txt
+Assets/mou1-167abfbe90bd160c.jpeg
+Assets/mou2-e527094ff149f3f5.jpeg
+Assets/mou3-7555921bb73506bc.jpeg
+Assets/2067562439948808366-6aa4b4500bb7b7b2</t>
+  </si>
+  <si>
+    <t>News and Goverment Sources/EVC-005_01_IMG_2121-7b6e3c30fde93c7c.png
+News and Goverment Sources/EVC-005_02_IMG_2122-8e3e775c9143519c.png
+News and Goverment Sources/EVC-005_03_IMG_2123-ff4e4bcfd71229ac.png
+News and Goverment Sources/EVC-005_04_IMG_3526-7bd2193fb2ae45ba.jpg
+News and Goverment Sources/EVC-005_05_IMG_3524-8eaf21a3cadadac4.jpg
+News and Goverment Sources/EVC-005_06_IMG_3482-ca26986df53d8d39.png
+News and Goverment Sources/EVC-005_07_message-22503970b78b530b.txt
+News and Goverment Sources/EVC-005_08_mou1-167abfbe90bd160c.jpeg
+News and Goverment Sources/EVC-005_09_mou2-e527094ff149f3f5.jpeg
+News and Goverment Sources/EVC-005_10_mou3-7555921bb73506bc.jpeg
+News and Goverment Sources/EVC-005_11_2067562439948808366-6aa4b4500bb7b7b2.png</t>
+  </si>
+  <si>
+    <t>Submitted MoU document pages, official-release related material, and formal-peace-negotiation context used to argue that the MoU was not a definitive permanent peace agreement by the June 15 deadline.</t>
+  </si>
+  <si>
+    <t>ll / 5010 / 传其常情</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517168284602994829
+https://discord.com/channels/1516872609105711124/1517091731236192418/1519082494048338152
+https://discord.com/channels/1516872609105711124/1517091731236192418/1520466923865903264</t>
+  </si>
+  <si>
+    <t>MoU text / government-source review / rule condition</t>
+  </si>
+  <si>
+    <t>Preserves supporting materials for the argument that the MoU contemplated future final-deal steps, temporary periods, or later publication rather than a qualifying permanent peace deal by June 15.</t>
+  </si>
+  <si>
+    <t>RULE-NO-002; RULE-NO-005; RULE-NO-006; RULE-NO-007</t>
+  </si>
+  <si>
+    <t>News and Goverment Sources/EVC-005_01_IMG_2121-7b6e3c30fde93c7c.png: c16a07bcd88dbd92f1851559856548fa7b5798eab7d126f1a3335db3a0729bc0
+News and Goverment Sources/EVC-005_02_IMG_2122-8e3e775c9143519c.png: 2f06262ec2ff11a5fe0834c66a8b929b4540bf89c0817e204046e95655bee8b2
+News and Goverment Sources/EVC-005_03_IMG_2123-ff4e4bcfd71229ac.png: 199579dd1678b7a0884bf39c171fbb213f907b284289d56060a66113c30ef76d
+News and Goverment Sources/EVC-005_04_IMG_3526-7bd2193fb2ae45ba.jpg: 111a620c0fec3d1751942cd827d3d72e551895aadbb7341a91ba44a307ac777e
+News and Goverment Sources/EVC-005_05_IMG_3524-8eaf21a3cadadac4.jpg: aa5632a5f9747694b59bf0b64c182c263931c74229ecac1b1c7678802273dc6a
+News and Goverment Sources/EVC-005_06_IMG_3482-ca26986df53d8d39.png: 4bcf4bb926396f33fac2d2895ea874f6a95ace5bda589d61225a804bea3ac1bc
+News and Goverment Sources/EVC-005_07_message-22503970b78b530b.txt: 6c48c497691c2b52c6190c301a8fcabb226712ede36cde59429f1cbab17b0264
+News and Goverment Sources/EVC-005_08_mou1-167abfbe90bd160c.jpeg: ff2becf49c03010d65c1182ee53e1eae03da02dbf7fec1983320a86a5a220bcf
+News and Goverment Sources/EVC-005_09_mou2-e527094ff149f3f5.jpeg: bc7deece6d967cef0faf8954fc2c018451555324957f36497bd7dd16de4df5f2
+News and Goverment Sources/EVC-005_10_mou3-7555921bb73506bc.jpeg: 6c16a9053b3b2f529ca291606f98421cc0d25ca08cf76c77c54d86de82cb7e30
+News and Goverment Sources/EVC-005_11_2067562439948808366-6aa4b4500bb7b7b2.png: 6fbff0e9d84068bf5160c272d5457bac4d60c8d7bc0426e8a2182515f819afc0</t>
+  </si>
+  <si>
+    <t>Includes screenshots and text file submitted in Discord. Source authenticity and translations should be reviewed by counsel or a subject-matter expert.</t>
+  </si>
+  <si>
+    <t>EVC-006</t>
+  </si>
+  <si>
+    <t>Assets/image-dbd98beb30ddb682.png
+Assets/image-82d4deb7c2c182c4.png
+Assets/Benni_UMA_Discord_owner_appearance-23df4b07753333f9.rar</t>
+  </si>
+  <si>
+    <t>UMA disputers coordination/EVC-006_01_image-dbd98beb30ddb682.png
+UMA disputers coordination/EVC-006_02_image-82d4deb7c2c182c4.png
+UMA disputers coordination/EVC-006_03_Benni_UMA_Discord_owner_appearance-23df4b07753333f9.rar</t>
+  </si>
+  <si>
+    <t>UMA-related coordination and voting-power context, including UMA.rocks screenshots and a submitted archive of Benni / UMA Discord owner appearance screenshots during disputes.</t>
+  </si>
+  <si>
+    <t>Sami / unknown forwarded submitter</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517136219807416320
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517138854220660756</t>
+  </si>
+  <si>
+    <t>UMA voting process / dispute coordination context</t>
+  </si>
+  <si>
+    <t>Supports review of UMA voting centralization, delegated voting services, and influential participant presence during dispute discussions.</t>
+  </si>
+  <si>
+    <t>EV-023; DCE-006; DCE-007; DCE-010; DCE-011; DCE-014; DCE-015</t>
+  </si>
+  <si>
+    <t>UMA disputers coordination/EVC-006_01_image-dbd98beb30ddb682.png: b4df64c790601905a6345e242b127f406107c12a871d23d131274f63c978587c
+UMA disputers coordination/EVC-006_02_image-82d4deb7c2c182c4.png: bb93da049f1b30c24c77ca682de8f8b5b1cf42e07425769972020d5cc7dae6f3
+UMA disputers coordination/EVC-006_03_Benni_UMA_Discord_owner_appearance-23df4b07753333f9.rar: a51d42a76c0febc73d6878426285c867bf4b6ee7297b4f178feca6c656924548</t>
+  </si>
+  <si>
+    <t>The RAR is preserved as submitted. It should be unpacked and reviewed separately before each internal screenshot is cited individually.</t>
+  </si>
+  <si>
+    <t>EVC-007</t>
+  </si>
+  <si>
+    <t>Assets/image-cc785c9e02ccf7d9.png
+Assets/image-4cae564b791be8ab.png
+Assets/image-ac0b79efd1165b13.png
+Assets/image-525ba283d6165a2f.png
+Assets/image-8bbc2d9eb6d0993a.png</t>
+  </si>
+  <si>
+    <t>Trade History/EVC-007_01_image-cc785c9e02ccf7d9.png
+Trade History/EVC-007_02_image-4cae564b791be8ab.png
+Trade History/EVC-007_03_image-ac0b79efd1165b13.png
+Trade History/EVC-007_04_image-525ba283d6165a2f.png
+Trade History/EVC-007_05_image-8bbc2d9eb6d0993a.png</t>
+  </si>
+  <si>
+    <t>Screenshots submitted as possible price-action evidence showing large YES-side trading or price movement near the disputed resolution period.</t>
+  </si>
+  <si>
+    <t>Sami</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517140427575267438</t>
+  </si>
+  <si>
+    <t>Possible price movement / final review optics</t>
+  </si>
+  <si>
+    <t>May support a forensic review of whether large YES-side traders moved market prices toward 100 percent before or during final review.</t>
+  </si>
+  <si>
+    <t>TRADE-001; TRADE-002; ACTIVITY-001; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>Trade History/EVC-007_01_image-cc785c9e02ccf7d9.png: 9c648fad6d1ac4c314633089b609b3264641ffa2967345341c61aa7b4a4a62b8
+Trade History/EVC-007_02_image-4cae564b791be8ab.png: ae2129fb6e5ba4d0be76b9c9b47f70e0add5b50dedffd525ab2afe2b9fb65396
+Trade History/EVC-007_03_image-ac0b79efd1165b13.png: b4324dbc50f90ecb8f7082b1bfaf230e9401e964b0e5daba86f613207a9acb5c
+Trade History/EVC-007_04_image-525ba283d6165a2f.png: 6237bb55f8c1d4bb01b2ccf0366c1c0c8e9da417ca1f0922f1265c3047bebeaf
+Trade History/EVC-007_05_image-8bbc2d9eb6d0993a.png: 5b425bdfa9c0a152d5eb87c95f4134f3f8ff96eb5a05ec7ccfa965f068dcd65c</t>
+  </si>
+  <si>
+    <t>The message labels this as circumstantial. Do not describe as manipulation without transaction-level verification and counsel review.</t>
+  </si>
+  <si>
+    <t>EVC-008</t>
+  </si>
+  <si>
+    <t>Assets/image0-4386278a36442e8c.jpg
+Assets/image0-02e670cd80f5b8e5.jpg
+Assets/image0-7e9659a1d5c8a64c.jpg
+Assets/image0-fd1b4d7f9a804c38.jpg
+Assets/2C5867BF-F37B-4CE6-B39C-3CBF2B7B0B56-9625bd9d737af218.jpg
+Assets/IMG_3478-fbb828b1cb7d3aeb.png
+Assets/IMG_3477-6148232d1b947e41.png
+Assets/IMG_3476-c2d7895961d089ab.png
+Assets/image-0d369a9e50bf8c0e.png</t>
+  </si>
+  <si>
+    <t>Insider Trading News/EVC-008_01_image0-4386278a36442e8c.jpg
+Insider Trading News/EVC-008_02_image0-02e670cd80f5b8e5.jpg
+Insider Trading News/EVC-008_03_image0-7e9659a1d5c8a64c.jpg
+Insider Trading News/EVC-008_04_image0-fd1b4d7f9a804c38.jpg
+Insider Trading News/EVC-008_05_2C5867BF-F37B-4CE6-B39C-3CBF2B7B0B56-9625bd9d737af218.jpg
+Insider Trading News/EVC-008_06_IMG_3478-fbb828b1cb7d3aeb.png
+Insider Trading News/EVC-008_07_IMG_3477-6148232d1b947e41.png
+Insider Trading News/EVC-008_08_IMG_3476-c2d7895961d089ab.png
+Insider Trading News/EVC-008_09_image-0d369a9e50bf8c0e.png</t>
+  </si>
+  <si>
+    <t>Screenshots submitted as pattern evidence concerning recurring Polymarket users or wallets such as Car, Denizz, wan123, 18, and related accounts across controversial markets.</t>
+  </si>
+  <si>
+    <t>Teh Golden Buddha / Sr Francisco / unknown forwarded submitter</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517382199135965284
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517383020515033198
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517383397662658731
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517515687512244324
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517515874796441743
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517516703615946842
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517538849666895894</t>
+  </si>
+  <si>
+    <t>Pattern evidence / related markets / recurring participant review</t>
+  </si>
+  <si>
+    <t>May help identify recurring actors or wallets appearing on favorable sides of multiple controversial markets, subject to independent wallet and trade-history verification.</t>
+  </si>
+  <si>
+    <t>IR-RAW-001; IR-RAW-009; TRADE-001; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>Insider Trading News/EVC-008_01_image0-4386278a36442e8c.jpg: a1fd99535021db96b6c0b93cb1b5d2219d721c789cc9f54f506a094bf2dd757d
+Insider Trading News/EVC-008_02_image0-02e670cd80f5b8e5.jpg: 805c27c9bbc2ecadf5e1583240702c047a6cc12673270c3a2a3936fb494470b2
+Insider Trading News/EVC-008_03_image0-7e9659a1d5c8a64c.jpg: 1fb749e19f7f94499270fdf6dd40b0aba29d41429a9317ebc916b63eb05b0bbb
+Insider Trading News/EVC-008_04_image0-fd1b4d7f9a804c38.jpg: c5147761cd9f822cc4de00abdb0c6dfd610e4b0f8e6803b14c763360c1bde81a
+Insider Trading News/EVC-008_05_2C5867BF-F37B-4CE6-B39C-3CBF2B7B0B56-9625bd9d737af218.jpg: 0441e520a184eb78c5a1059eeda6aa1b07fd1014c22222a0b669ce3e23f49c25
+Insider Trading News/EVC-008_06_IMG_3478-fbb828b1cb7d3aeb.png: 2b36930283c6c5d671b2b41d030c37274af938bc69b91780b3fc0d8c6cdd99c7
+Insider Trading News/EVC-008_07_IMG_3477-6148232d1b947e41.png: 04704d631da9162893eab371afebd18b38af0d5c46ff0cb90f6ce8d00a401663
+Insider Trading News/EVC-008_08_IMG_3476-c2d7895961d089ab.png: 80bddbcd3ebda2d9d1cf7179afe128f5d0f4d182b8d31c7c235768fc390921e5
+Insider Trading News/EVC-008_09_image-0d369a9e50bf8c0e.png: 01b86508d5065ab530d823f8142a9bc0886a5078bced7f3fd60e6e620ec1e356</t>
+  </si>
+  <si>
+    <t>This is pattern and lead evidence only. It should be connected to wallet-level data before being used as actor-specific proof.</t>
+  </si>
+  <si>
+    <t>EVC-009</t>
+  </si>
+  <si>
+    <t>Assets/HLLTrB8aAAAyh5A-e39071187a5290cc.jpg_large
+Assets/HLKxQ77bcAAjuw5-c34c369fe55830ee.jpg_large</t>
+  </si>
+  <si>
+    <t>Insider Trading News/EVC-009_01_HLLTrB8aAAAyh5A-e39071187a5290cc.jpg_large
+Insider Trading News/EVC-009_02_HLKxQ77bcAAjuw5-c34c369fe55830ee.jpg_large</t>
+  </si>
+  <si>
+    <t>X/Twitter public breakdown screenshots concerning the “Car” Polymarket account and the YES-side narrative in the US-Iran permanent peace deal dispute.</t>
+  </si>
+  <si>
+    <t>Teh Golden Buddha / unknown</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517529159885258774
+https://discord.com/channels/1516872609105711124/1517091731236192418/1517530187028496404</t>
+  </si>
+  <si>
+    <t>Public analysis / actor-specific lead</t>
+  </si>
+  <si>
+    <t>Preserves public analysis links and preview images that may assist counsel in identifying public allegations and leads for further verification.</t>
+  </si>
+  <si>
+    <t>EVC-008; IR-RAW-001; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>Insider Trading News/EVC-009_01_HLLTrB8aAAAyh5A-e39071187a5290cc.jpg_large: 569a1ee12f646660f4952ce33ba39ec84c2fe3398bb480346d18536e2efd1340
+Insider Trading News/EVC-009_02_HLKxQ77bcAAjuw5-c34c369fe55830ee.jpg_large: d68e69254b0e713e2c5989e95c81acf4dd71583379154e45fd680802223b6a94</t>
+  </si>
+  <si>
+    <t>Use as public-source lead material only. Verify the underlying X posts and any wallet/account assertions before relying on them.</t>
+  </si>
+  <si>
+    <t>EVC-010</t>
+  </si>
+  <si>
+    <t>Assets/Polymarket_-_US-Iran_peace_deal_-_objectio-0db6194abd29ad43.docx</t>
+  </si>
+  <si>
+    <t>Polymarket Statements/EVC-010_01_Polymarket_-_US-Iran_peace_deal_-_objectio-0db6194abd29ad43.docx</t>
+  </si>
+  <si>
+    <t>Community member objection email to Polymarket concerning the US-Iran permanent peace agreement by June 15 market, including argumentation and reference links.</t>
+  </si>
+  <si>
+    <t>Matesovič</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1517199304383664322</t>
+  </si>
+  <si>
+    <t>Notice to Polymarket / objection arguments</t>
+  </si>
+  <si>
+    <t>May support notice, dispute history, and contemporaneous claimant arguments delivered or prepared for Polymarket.</t>
+  </si>
+  <si>
+    <t>PM-STMT-001; PM-STMT-002; PM-RULE-001</t>
+  </si>
+  <si>
+    <t>Polymarket Statements/EVC-010_01_Polymarket_-_US-Iran_peace_deal_-_objectio-0db6194abd29ad43.docx: e22612dfe3f1c149266e710acbe9dd9a803a256bbf310dc294e5323000569772</t>
+  </si>
+  <si>
+    <t>Treat as user-submitted correspondence. Counsel should verify whether and when it was sent to Polymarket.</t>
+  </si>
+  <si>
+    <t>EVC-011</t>
+  </si>
+  <si>
+    <t>Assets/Investigation_Report-3857a64b9ca49b13.md</t>
+  </si>
+  <si>
+    <t>Insider Trading News/EVC-011_01_Investigation_Report-3857a64b9ca49b13.md</t>
+  </si>
+  <si>
+    <t>User-submitted forensic investigation report alleging a 19-wallet cluster, shared funders, synchronized trades, and large BUY YES exposure.</t>
+  </si>
+  <si>
+    <t>Teh Golden Buddha</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1518059241506738286</t>
+  </si>
+  <si>
+    <t>Wallet cluster / forensic analysis lead</t>
+  </si>
+  <si>
+    <t>Supports counsel and expert review of the wallet-cluster theory and potential shared-funder or synchronized-trading patterns.</t>
+  </si>
+  <si>
+    <t>IR-RAW-001; IR-RAW-005; IR-RAW-006; APP-CONFLICT-001; SUS-001; SUS-010</t>
+  </si>
+  <si>
+    <t>Insider Trading News/EVC-011_01_Investigation_Report-3857a64b9ca49b13.md: e413e64778b0704b858799835ec777fb25a386f227836b7bebd750d82b19ab09</t>
+  </si>
+  <si>
+    <t>Derived analysis only. Underlying raw data should be cross-checked against existing IR-RAW, APP, and SUS exhibits.</t>
+  </si>
+  <si>
+    <t>EVC-012</t>
+  </si>
+  <si>
+    <t>Assets/uma_perma_peace_deal_june_15_thread-5be3016ed216414a.txt
+Assets/screencapture-oracle-uma-xyz-2026-06-16-12-a15f15c07ed09435.png</t>
+  </si>
+  <si>
+    <t>UMA disputers coordination/EVC-012_01_uma_perma_peace_deal_june_15_thread-5be3016ed216414a.txt
+UMA disputers coordination/EVC-012_02_screencapture-oracle-uma-xyz-2026-06-16-12-a15f15c07ed09435.png</t>
+  </si>
+  <si>
+    <t>Copied text of the UMA Discord thread for the June 15 US-Iran permanent peace deal dispute, plus a UMA oracle page capture showing rules and related addresses.</t>
+  </si>
+  <si>
+    <t>Teh Golden Buddha / Matesovič</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1518128765765419059
+https://discord.com/channels/1516872609105711124/1517091731236192418/1518178883063513259</t>
+  </si>
+  <si>
+    <t>UMA dispute thread / oracle page identity</t>
+  </si>
+  <si>
+    <t>Preserves an additional text copy of the UMA discussion and a large UMA oracle screenshot that may support market-to-UMA identity and dispute-context review.</t>
+  </si>
+  <si>
+    <t>DCE-006; DCE-007; UMA-UI-001; UMA-UI-002; UMA-004</t>
+  </si>
+  <si>
+    <t>UMA disputers coordination/EVC-012_01_uma_perma_peace_deal_june_15_thread-5be3016ed216414a.txt: 280022674e5702b8a9a1d37fc40002b939d16d61f76a8d54102b7123efb60dd4
+UMA disputers coordination/EVC-012_02_screencapture-oracle-uma-xyz-2026-06-16-12-a15f15c07ed09435.png: f78d9d44025862b302263f478b6248da9dcdc5d86d71480a13d7cfb794697710</t>
+  </si>
+  <si>
+    <t>The text file is a copy-paste capture, not a native export. Use the authenticated JSON/HTML exports as primary records where available.</t>
+  </si>
+  <si>
+    <t>EVC-013</t>
+  </si>
+  <si>
+    <t>Assets/image-7ce372636fe41498.png
+Assets/image-54b8727d0b2fb06e.png
+Assets/image-ff15991947d38402.png
+Assets/image-82bea94596e90bc1.png
+Assets/image-91ea74ac2cab894a.png</t>
+  </si>
+  <si>
+    <t>Trade History/EVC-013_01_image-7ce372636fe41498.png
+Trade History/EVC-013_02_image-54b8727d0b2fb06e.png
+Trade History/EVC-013_03_image-ff15991947d38402.png
+Trade History/EVC-013_04_image-82bea94596e90bc1.png
+Trade History/EVC-013_05_image-91ea74ac2cab894a.png</t>
+  </si>
+  <si>
+    <t>Additional screenshots from a Polymarket analyzer / graph workflow showing trader, funder, and event relationships for the related Iran markets.</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1518265917056880807
+https://discord.com/channels/1516872609105711124/1517091731236192418/1518276672284131388</t>
+  </si>
+  <si>
+    <t>Wallet graph / market analyzer output</t>
+  </si>
+  <si>
+    <t>May supplement the existing app and PolyAudit exhibits by preserving additional visual outputs related to trader/funder mapping.</t>
+  </si>
+  <si>
+    <t>APP-001; APP-002; APP-003; APP-005; APP-006; APP-CONFLICT-001</t>
+  </si>
+  <si>
+    <t>Trade History/EVC-013_01_image-7ce372636fe41498.png: e034687fc156f96f24e174185347ec47fa827916e2b776ca265b354dd1b3cbc2
+Trade History/EVC-013_02_image-54b8727d0b2fb06e.png: db758c71efaa1f30312af4c31428fbe01b9bebee3a932b745a2eb2eb16c3dd57
+Trade History/EVC-013_03_image-ff15991947d38402.png: 2c30d037c56d7075861acf3407d2a9e622deabc4bd366bfa8a63c54e66d59cce
+Trade History/EVC-013_04_image-82bea94596e90bc1.png: 7820750c755dc2ff4a5811f1e9b63b89e2b9a1c4a0db794a62c54327ef8498fc
+Trade History/EVC-013_05_image-91ea74ac2cab894a.png: ed19aa7251458f6d3824b38b426f57ce79ce1949b26230c9847da849aec1d693</t>
+  </si>
+  <si>
+    <t>Visual outputs should be tied back to raw app data and underlying on-chain records before being used as proof.</t>
+  </si>
+  <si>
+    <t>EVC-014</t>
+  </si>
+  <si>
+    <t>Assets/Screenshot_2026-06-21_at_14.48.41-664896eae72a7bf8.png</t>
+  </si>
+  <si>
+    <t>Market Page/EVC-014_01_Screenshot_2026-06-21_at_14.48.41-664896eae72a7bf8.png</t>
+  </si>
+  <si>
+    <t>Screenshot submitted as “the three Iran related markets,” showing related Polymarket Iran market context.</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1518255952736948387</t>
+  </si>
+  <si>
+    <t>May help show the market group and related date markets connected to the damages and cross-market analysis.</t>
+  </si>
+  <si>
+    <t>PM-MKT-001; LOSS-001; LOSS-002; TRADE-002</t>
+  </si>
+  <si>
+    <t>Market Page/EVC-014_01_Screenshot_2026-06-21_at_14.48.41-664896eae72a7bf8.png: e276f80a96323c96db0c49693ba27d6139501944f2e828b5cf5ee3d2a6963f39</t>
+  </si>
+  <si>
+    <t>Corroborating screenshot only. Use underlying Polymarket metadata and loss files for final market identification.</t>
+  </si>
+  <si>
+    <t>EVC-015</t>
+  </si>
+  <si>
+    <t>Assets/2070179486335983686-42adcacf23bb83f3
+Assets/2069501943551086870-c38b5c77f46b0fe9
+Assets/gettyimages-2283273999-7d0ad2ab680d884c.jpg
+Assets/2070556848311222575-895321ab2d7ab9b5
+Assets/2069436413599465776-b6a5066f2de44b2d</t>
+  </si>
+  <si>
+    <t>Insider Trading News/EVC-015_01_2070179486335983686-42adcacf23bb83f3.png
+Insider Trading News/EVC-015_02_2069501943551086870-c38b5c77f46b0fe9.png
+Insider Trading News/EVC-015_03_gettyimages-2283273999-7d0ad2ab680d884c.jpg
+Insider Trading News/EVC-015_04_2070556848311222575-895321ab2d7ab9b5.png
+Insider Trading News/EVC-015_05_2069436413599465776-b6a5066f2de44b2d.png</t>
+  </si>
+  <si>
+    <t>Selected public-media and public-commentary screenshots concerning Polymarket, the Iran dispute, UMA discussions, and broader public attention after the disputed resolution.</t>
+  </si>
+  <si>
+    <t>NΞY THΞ BΛSQUΞ 🐳 / LP / Kirk / Teh Golden Buddha / unknown</t>
+  </si>
+  <si>
+    <t>https://discord.com/channels/1516872609105711124/1517091731236192418/1519749307614363718
+https://discord.com/channels/1516872609105711124/1517091731236192418/1519919007313170465
+https://discord.com/channels/1516872609105711124/1517091731236192418/1520247929091264583
+https://discord.com/channels/1516872609105711124/1517091731236192418/1520256995142402159
+https://discord.com/channels/1516872609105711124/1517091731236192418/1520289460951056415</t>
+  </si>
+  <si>
+    <t>Public reporting / post-resolution scrutiny</t>
+  </si>
+  <si>
+    <t>Preserves public-facing follow-up material that may support media, regulatory, or context review, not the core rule-merits proof by itself.</t>
+  </si>
+  <si>
+    <t>PM-STMT-001; PM-STMT-002; DCE-010; DCE-011</t>
+  </si>
+  <si>
+    <t>Insider Trading News/EVC-015_01_2070179486335983686-42adcacf23bb83f3.png: f91f3c766d2689c2287384f996e4bbbca3598909048cb3ddc1327b70e19c3df0
+Insider Trading News/EVC-015_02_2069501943551086870-c38b5c77f46b0fe9.png: bd17e350de2a43d8a02d09b0e7385a06c4afdbe7cee1a7a67c134cc86b294833
+Insider Trading News/EVC-015_03_gettyimages-2283273999-7d0ad2ab680d884c.jpg: 2f38f92e6d37d07613f7a49241f07111cb9ebc0fcaa7d81ca1d4da973a682d56
+Insider Trading News/EVC-015_04_2070556848311222575-895321ab2d7ab9b5.png: 0a97de83bf4d52279e8b261a8a4aca95fd82e9c065a4b823188fa397eb2e704f
+Insider Trading News/EVC-015_05_2069436413599465776-b6a5066f2de44b2d.png: 9a910d009cdda648120e245b4f654a530ec11428d36941d0fcf369f5d5683223</t>
+  </si>
+  <si>
+    <t>Post-resolution public commentary should be separated from the core June 15 rule-condition proof.</t>
   </si>
 </sst>
 </file>
@@ -3317,7 +4436,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:S984" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:S981" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="19">
     <tableColumn name="Evidence ID" id="1"/>
     <tableColumn name="Evidence category" id="2"/>
@@ -9684,786 +10803,2010 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="15"/>
-      <c r="B105" s="16"/>
-      <c r="C105" s="16"/>
-      <c r="D105" s="16"/>
-      <c r="E105" s="11"/>
-      <c r="F105" s="11"/>
-      <c r="G105" s="16"/>
-      <c r="H105" s="16"/>
-      <c r="I105" s="11"/>
-      <c r="J105" s="11"/>
-      <c r="K105" s="11"/>
-      <c r="L105" s="16"/>
-      <c r="M105" s="11"/>
-      <c r="N105" s="11"/>
-      <c r="O105" s="11"/>
-      <c r="P105" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q105" s="11"/>
-      <c r="R105" s="11"/>
-      <c r="S105" s="11"/>
+      <c r="A105" s="4" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C105" s="7" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>1004</v>
+      </c>
+      <c r="E105" s="8" t="s">
+        <v>1005</v>
+      </c>
+      <c r="F105" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G105" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H105" s="13" t="s">
+        <v>1008</v>
+      </c>
+      <c r="I105" s="14">
+        <v>46123.0</v>
+      </c>
+      <c r="J105" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K105" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L105" s="7" t="s">
+        <v>1009</v>
+      </c>
+      <c r="M105" s="8" t="s">
+        <v>1010</v>
+      </c>
+      <c r="N105" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O105" s="8" t="s">
+        <v>1011</v>
+      </c>
+      <c r="P105" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q105" s="8" t="s">
+        <v>1012</v>
+      </c>
+      <c r="R105" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S105" s="8" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="15"/>
-      <c r="B106" s="16"/>
-      <c r="C106" s="16"/>
-      <c r="D106" s="16"/>
-      <c r="E106" s="11"/>
-      <c r="F106" s="11"/>
-      <c r="G106" s="16"/>
-      <c r="H106" s="16"/>
-      <c r="I106" s="11"/>
-      <c r="J106" s="11"/>
-      <c r="K106" s="11"/>
-      <c r="L106" s="16"/>
-      <c r="M106" s="11"/>
-      <c r="N106" s="11"/>
-      <c r="O106" s="11"/>
-      <c r="P106" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q106" s="11"/>
-      <c r="R106" s="11"/>
-      <c r="S106" s="11"/>
+      <c r="A106" s="4" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C106" s="7" t="s">
+        <v>1015</v>
+      </c>
+      <c r="D106" s="7" t="s">
+        <v>1016</v>
+      </c>
+      <c r="E106" s="8" t="s">
+        <v>1017</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G106" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H106" s="13" t="s">
+        <v>1008</v>
+      </c>
+      <c r="I106" s="14">
+        <v>46123.0</v>
+      </c>
+      <c r="J106" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K106" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L106" s="7" t="s">
+        <v>1009</v>
+      </c>
+      <c r="M106" s="8" t="s">
+        <v>1018</v>
+      </c>
+      <c r="N106" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O106" s="8" t="s">
+        <v>1019</v>
+      </c>
+      <c r="P106" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q106" s="8" t="s">
+        <v>1020</v>
+      </c>
+      <c r="R106" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S106" s="8" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="15"/>
-      <c r="B107" s="16"/>
-      <c r="C107" s="16"/>
-      <c r="D107" s="16"/>
-      <c r="E107" s="11"/>
-      <c r="F107" s="11"/>
-      <c r="G107" s="16"/>
-      <c r="H107" s="16"/>
-      <c r="I107" s="11"/>
-      <c r="J107" s="11"/>
-      <c r="K107" s="11"/>
-      <c r="L107" s="16"/>
-      <c r="M107" s="11"/>
-      <c r="N107" s="11"/>
-      <c r="O107" s="11"/>
-      <c r="P107" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q107" s="11"/>
-      <c r="R107" s="11"/>
-      <c r="S107" s="11"/>
+      <c r="A107" s="4" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C107" s="7" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D107" s="7" t="s">
+        <v>1023</v>
+      </c>
+      <c r="E107" s="8" t="s">
+        <v>1024</v>
+      </c>
+      <c r="F107" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G107" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H107" s="13" t="s">
+        <v>1025</v>
+      </c>
+      <c r="I107" s="14">
+        <v>45840.0</v>
+      </c>
+      <c r="J107" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K107" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L107" s="7" t="s">
+        <v>1026</v>
+      </c>
+      <c r="M107" s="8" t="s">
+        <v>1027</v>
+      </c>
+      <c r="N107" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O107" s="8" t="s">
+        <v>1028</v>
+      </c>
+      <c r="P107" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q107" s="8" t="s">
+        <v>1029</v>
+      </c>
+      <c r="R107" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S107" s="8" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="15"/>
-      <c r="B108" s="16"/>
-      <c r="C108" s="16"/>
-      <c r="D108" s="16"/>
-      <c r="E108" s="11"/>
-      <c r="F108" s="11"/>
-      <c r="G108" s="16"/>
-      <c r="H108" s="16"/>
-      <c r="I108" s="11"/>
-      <c r="J108" s="11"/>
-      <c r="K108" s="11"/>
-      <c r="L108" s="16"/>
-      <c r="M108" s="11"/>
-      <c r="N108" s="11"/>
-      <c r="O108" s="11"/>
-      <c r="P108" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q108" s="11"/>
-      <c r="R108" s="11"/>
-      <c r="S108" s="11"/>
+      <c r="A108" s="4" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C108" s="7" t="s">
+        <v>1031</v>
+      </c>
+      <c r="D108" s="7" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E108" s="8" t="s">
+        <v>1033</v>
+      </c>
+      <c r="F108" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G108" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H108" s="13" t="s">
+        <v>1025</v>
+      </c>
+      <c r="I108" s="14">
+        <v>45840.0</v>
+      </c>
+      <c r="J108" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K108" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L108" s="7" t="s">
+        <v>1026</v>
+      </c>
+      <c r="M108" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="N108" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O108" s="8" t="s">
+        <v>1035</v>
+      </c>
+      <c r="P108" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q108" s="8" t="s">
+        <v>1036</v>
+      </c>
+      <c r="R108" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S108" s="8" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="15"/>
-      <c r="B109" s="16"/>
-      <c r="C109" s="16"/>
-      <c r="D109" s="16"/>
-      <c r="E109" s="11"/>
-      <c r="F109" s="11"/>
-      <c r="G109" s="16"/>
-      <c r="H109" s="16"/>
-      <c r="I109" s="11"/>
-      <c r="J109" s="11"/>
-      <c r="K109" s="11"/>
-      <c r="L109" s="16"/>
-      <c r="M109" s="11"/>
-      <c r="N109" s="11"/>
-      <c r="O109" s="11"/>
-      <c r="P109" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q109" s="11"/>
-      <c r="R109" s="11"/>
-      <c r="S109" s="11"/>
+      <c r="A109" s="4" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D109" s="7" t="s">
+        <v>1039</v>
+      </c>
+      <c r="E109" s="8" t="s">
+        <v>1040</v>
+      </c>
+      <c r="F109" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G109" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H109" s="13" t="s">
+        <v>1041</v>
+      </c>
+      <c r="I109" s="14">
+        <v>46187.0</v>
+      </c>
+      <c r="J109" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K109" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L109" s="7" t="s">
+        <v>1042</v>
+      </c>
+      <c r="M109" s="8" t="s">
+        <v>1043</v>
+      </c>
+      <c r="N109" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O109" s="8" t="s">
+        <v>1044</v>
+      </c>
+      <c r="P109" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q109" s="8" t="s">
+        <v>1045</v>
+      </c>
+      <c r="R109" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S109" s="8" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="15"/>
-      <c r="B110" s="16"/>
-      <c r="C110" s="16"/>
-      <c r="D110" s="16"/>
-      <c r="E110" s="11"/>
-      <c r="F110" s="11"/>
-      <c r="G110" s="16"/>
-      <c r="H110" s="16"/>
-      <c r="I110" s="11"/>
-      <c r="J110" s="11"/>
-      <c r="K110" s="11"/>
-      <c r="L110" s="16"/>
-      <c r="M110" s="11"/>
-      <c r="N110" s="11"/>
-      <c r="O110" s="11"/>
-      <c r="P110" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q110" s="11"/>
-      <c r="R110" s="11"/>
-      <c r="S110" s="11"/>
+      <c r="A110" s="4" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C110" s="7" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D110" s="7" t="s">
+        <v>1048</v>
+      </c>
+      <c r="E110" s="8" t="s">
+        <v>1049</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G110" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H110" s="13" t="s">
+        <v>1041</v>
+      </c>
+      <c r="I110" s="14">
+        <v>46187.0</v>
+      </c>
+      <c r="J110" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K110" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L110" s="7" t="s">
+        <v>1042</v>
+      </c>
+      <c r="M110" s="8" t="s">
+        <v>1050</v>
+      </c>
+      <c r="N110" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O110" s="8" t="s">
+        <v>1051</v>
+      </c>
+      <c r="P110" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q110" s="8" t="s">
+        <v>1052</v>
+      </c>
+      <c r="R110" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S110" s="8" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="15"/>
-      <c r="B111" s="16"/>
-      <c r="C111" s="16"/>
-      <c r="D111" s="16"/>
-      <c r="E111" s="11"/>
-      <c r="F111" s="11"/>
-      <c r="G111" s="16"/>
-      <c r="H111" s="16"/>
-      <c r="I111" s="11"/>
-      <c r="J111" s="11"/>
-      <c r="K111" s="11"/>
-      <c r="L111" s="16"/>
-      <c r="M111" s="11"/>
-      <c r="N111" s="11"/>
-      <c r="O111" s="11"/>
-      <c r="P111" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q111" s="11"/>
-      <c r="R111" s="11"/>
-      <c r="S111" s="11"/>
+      <c r="A111" s="4" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C111" s="7" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D111" s="7" t="s">
+        <v>1055</v>
+      </c>
+      <c r="E111" s="8" t="s">
+        <v>1056</v>
+      </c>
+      <c r="F111" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G111" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H111" s="13" t="s">
+        <v>1025</v>
+      </c>
+      <c r="I111" s="14">
+        <v>45840.0</v>
+      </c>
+      <c r="J111" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K111" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L111" s="7" t="s">
+        <v>1026</v>
+      </c>
+      <c r="M111" s="8" t="s">
+        <v>1057</v>
+      </c>
+      <c r="N111" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O111" s="8" t="s">
+        <v>1058</v>
+      </c>
+      <c r="P111" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q111" s="8" t="s">
+        <v>1029</v>
+      </c>
+      <c r="R111" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S111" s="8" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="112">
-      <c r="A112" s="15"/>
-      <c r="B112" s="16"/>
-      <c r="C112" s="16"/>
-      <c r="D112" s="16"/>
-      <c r="E112" s="11"/>
-      <c r="F112" s="11"/>
-      <c r="G112" s="16"/>
-      <c r="H112" s="16"/>
-      <c r="I112" s="11"/>
-      <c r="J112" s="11"/>
-      <c r="K112" s="11"/>
-      <c r="L112" s="16"/>
-      <c r="M112" s="11"/>
-      <c r="N112" s="11"/>
-      <c r="O112" s="11"/>
-      <c r="P112" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q112" s="11"/>
-      <c r="R112" s="11"/>
-      <c r="S112" s="11"/>
+      <c r="A112" s="4" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C112" s="7" t="s">
+        <v>1060</v>
+      </c>
+      <c r="D112" s="7" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E112" s="8" t="s">
+        <v>1062</v>
+      </c>
+      <c r="F112" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G112" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H112" s="13" t="s">
+        <v>1041</v>
+      </c>
+      <c r="I112" s="14">
+        <v>46187.0</v>
+      </c>
+      <c r="J112" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K112" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L112" s="7" t="s">
+        <v>1042</v>
+      </c>
+      <c r="M112" s="8" t="s">
+        <v>1063</v>
+      </c>
+      <c r="N112" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O112" s="8" t="s">
+        <v>1064</v>
+      </c>
+      <c r="P112" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q112" s="8" t="s">
+        <v>1045</v>
+      </c>
+      <c r="R112" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S112" s="8" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="113">
-      <c r="A113" s="15"/>
-      <c r="B113" s="16"/>
-      <c r="C113" s="16"/>
-      <c r="D113" s="16"/>
-      <c r="E113" s="11"/>
-      <c r="F113" s="11"/>
-      <c r="G113" s="16"/>
-      <c r="H113" s="16"/>
-      <c r="I113" s="11"/>
-      <c r="J113" s="11"/>
-      <c r="K113" s="11"/>
-      <c r="L113" s="16"/>
-      <c r="M113" s="11"/>
-      <c r="N113" s="11"/>
-      <c r="O113" s="11"/>
-      <c r="P113" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q113" s="11"/>
-      <c r="R113" s="11"/>
-      <c r="S113" s="11"/>
+      <c r="A113" s="4" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C113" s="7" t="s">
+        <v>1066</v>
+      </c>
+      <c r="D113" s="7" t="s">
+        <v>1067</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>1068</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G113" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H113" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I113" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="J113" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K113" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L113" s="7" t="s">
+        <v>1071</v>
+      </c>
+      <c r="M113" s="8" t="s">
+        <v>1072</v>
+      </c>
+      <c r="N113" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O113" s="8" t="s">
+        <v>1073</v>
+      </c>
+      <c r="P113" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q113" s="8" t="s">
+        <v>1074</v>
+      </c>
+      <c r="R113" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S113" s="8" t="s">
+        <v>1075</v>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="15"/>
-      <c r="B114" s="16"/>
-      <c r="C114" s="16"/>
-      <c r="D114" s="16"/>
-      <c r="E114" s="11"/>
-      <c r="F114" s="11"/>
-      <c r="G114" s="16"/>
-      <c r="H114" s="16"/>
-      <c r="I114" s="11"/>
-      <c r="J114" s="11"/>
-      <c r="K114" s="11"/>
-      <c r="L114" s="16"/>
-      <c r="M114" s="11"/>
-      <c r="N114" s="11"/>
-      <c r="O114" s="11"/>
-      <c r="P114" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q114" s="11"/>
-      <c r="R114" s="11"/>
-      <c r="S114" s="11"/>
+      <c r="A114" s="4" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C114" s="7" t="s">
+        <v>1077</v>
+      </c>
+      <c r="D114" s="7" t="s">
+        <v>1078</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>1079</v>
+      </c>
+      <c r="F114" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G114" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H114" s="13" t="s">
+        <v>1080</v>
+      </c>
+      <c r="I114" s="14">
+        <v>45842.0</v>
+      </c>
+      <c r="J114" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K114" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L114" s="7" t="s">
+        <v>1026</v>
+      </c>
+      <c r="M114" s="8" t="s">
+        <v>1081</v>
+      </c>
+      <c r="N114" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O114" s="8" t="s">
+        <v>1082</v>
+      </c>
+      <c r="P114" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q114" s="8" t="s">
+        <v>1083</v>
+      </c>
+      <c r="R114" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S114" s="8" t="s">
+        <v>1084</v>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" s="15"/>
-      <c r="B115" s="16"/>
-      <c r="C115" s="16"/>
-      <c r="D115" s="16"/>
-      <c r="E115" s="11"/>
-      <c r="F115" s="11"/>
-      <c r="G115" s="16"/>
-      <c r="H115" s="16"/>
-      <c r="I115" s="11"/>
-      <c r="J115" s="11"/>
-      <c r="K115" s="11"/>
-      <c r="L115" s="16"/>
-      <c r="M115" s="11"/>
-      <c r="N115" s="11"/>
-      <c r="O115" s="11"/>
-      <c r="P115" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q115" s="11"/>
-      <c r="R115" s="11"/>
-      <c r="S115" s="11"/>
+      <c r="A115" s="4" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C115" s="7" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D115" s="7" t="s">
+        <v>1087</v>
+      </c>
+      <c r="E115" s="8" t="s">
+        <v>1088</v>
+      </c>
+      <c r="F115" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G115" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H115" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I115" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="J115" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K115" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L115" s="7" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M115" s="8" t="s">
+        <v>1090</v>
+      </c>
+      <c r="N115" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O115" s="8" t="s">
+        <v>1091</v>
+      </c>
+      <c r="P115" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q115" s="8" t="s">
+        <v>1092</v>
+      </c>
+      <c r="R115" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S115" s="8" t="s">
+        <v>1093</v>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" s="15"/>
-      <c r="B116" s="16"/>
-      <c r="C116" s="16"/>
-      <c r="D116" s="16"/>
-      <c r="E116" s="11"/>
-      <c r="F116" s="11"/>
-      <c r="G116" s="16"/>
-      <c r="H116" s="16"/>
-      <c r="I116" s="11"/>
-      <c r="J116" s="11"/>
-      <c r="K116" s="11"/>
-      <c r="L116" s="16"/>
-      <c r="M116" s="11"/>
-      <c r="N116" s="11"/>
-      <c r="O116" s="11"/>
-      <c r="P116" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q116" s="11"/>
-      <c r="R116" s="11"/>
-      <c r="S116" s="11"/>
+      <c r="A116" s="4" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C116" s="7" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D116" s="7" t="s">
+        <v>1096</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>1097</v>
+      </c>
+      <c r="F116" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G116" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H116" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I116" s="14">
+        <v>46198.0</v>
+      </c>
+      <c r="J116" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K116" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L116" s="7" t="s">
+        <v>1098</v>
+      </c>
+      <c r="M116" s="8" t="s">
+        <v>1099</v>
+      </c>
+      <c r="N116" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O116" s="8" t="s">
+        <v>1100</v>
+      </c>
+      <c r="P116" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q116" s="8" t="s">
+        <v>1101</v>
+      </c>
+      <c r="R116" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S116" s="8" t="s">
+        <v>1102</v>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="15"/>
-      <c r="B117" s="16"/>
-      <c r="C117" s="16"/>
-      <c r="D117" s="16"/>
-      <c r="E117" s="11"/>
-      <c r="F117" s="11"/>
-      <c r="G117" s="16"/>
-      <c r="H117" s="16"/>
-      <c r="I117" s="11"/>
-      <c r="J117" s="11"/>
-      <c r="K117" s="11"/>
-      <c r="L117" s="16"/>
-      <c r="M117" s="11"/>
-      <c r="N117" s="11"/>
-      <c r="O117" s="11"/>
-      <c r="P117" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q117" s="11"/>
-      <c r="R117" s="11"/>
-      <c r="S117" s="11"/>
+      <c r="A117" s="4" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C117" s="7" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D117" s="7" t="s">
+        <v>1105</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>1106</v>
+      </c>
+      <c r="F117" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G117" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H117" s="13" t="s">
+        <v>1080</v>
+      </c>
+      <c r="I117" s="14">
+        <v>45842.0</v>
+      </c>
+      <c r="J117" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K117" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L117" s="7" t="s">
+        <v>1026</v>
+      </c>
+      <c r="M117" s="8" t="s">
+        <v>1107</v>
+      </c>
+      <c r="N117" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O117" s="8" t="s">
+        <v>1108</v>
+      </c>
+      <c r="P117" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q117" s="8" t="s">
+        <v>1109</v>
+      </c>
+      <c r="R117" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S117" s="8" t="s">
+        <v>1110</v>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="15"/>
-      <c r="B118" s="16"/>
-      <c r="C118" s="16"/>
-      <c r="D118" s="16"/>
-      <c r="E118" s="11"/>
-      <c r="F118" s="11"/>
-      <c r="G118" s="16"/>
-      <c r="H118" s="16"/>
-      <c r="I118" s="11"/>
-      <c r="J118" s="11"/>
-      <c r="K118" s="11"/>
-      <c r="L118" s="16"/>
-      <c r="M118" s="11"/>
-      <c r="N118" s="11"/>
-      <c r="O118" s="11"/>
-      <c r="P118" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q118" s="11"/>
-      <c r="R118" s="11"/>
-      <c r="S118" s="11"/>
+      <c r="A118" s="4" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>1112</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>1114</v>
+      </c>
+      <c r="F118" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G118" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H118" s="13" t="s">
+        <v>1115</v>
+      </c>
+      <c r="I118" s="14">
+        <v>45842.0</v>
+      </c>
+      <c r="J118" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K118" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L118" s="7" t="s">
+        <v>1026</v>
+      </c>
+      <c r="M118" s="8" t="s">
+        <v>1116</v>
+      </c>
+      <c r="N118" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O118" s="8" t="s">
+        <v>1117</v>
+      </c>
+      <c r="P118" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q118" s="8" t="s">
+        <v>1118</v>
+      </c>
+      <c r="R118" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S118" s="8" t="s">
+        <v>1119</v>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" s="15"/>
-      <c r="B119" s="16"/>
-      <c r="C119" s="16"/>
-      <c r="D119" s="16"/>
-      <c r="E119" s="11"/>
-      <c r="F119" s="11"/>
-      <c r="G119" s="16"/>
-      <c r="H119" s="16"/>
-      <c r="I119" s="11"/>
-      <c r="J119" s="11"/>
-      <c r="K119" s="11"/>
-      <c r="L119" s="16"/>
-      <c r="M119" s="11"/>
-      <c r="N119" s="11"/>
-      <c r="O119" s="11"/>
-      <c r="P119" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q119" s="11"/>
-      <c r="R119" s="11"/>
-      <c r="S119" s="11"/>
+      <c r="A119" s="4" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>1121</v>
+      </c>
+      <c r="D119" s="7" t="s">
+        <v>1122</v>
+      </c>
+      <c r="E119" s="8" t="s">
+        <v>1123</v>
+      </c>
+      <c r="F119" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G119" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H119" s="13" t="s">
+        <v>1124</v>
+      </c>
+      <c r="I119" s="14">
+        <v>46188.0</v>
+      </c>
+      <c r="J119" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K119" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L119" s="7" t="s">
+        <v>1042</v>
+      </c>
+      <c r="M119" s="8" t="s">
+        <v>1125</v>
+      </c>
+      <c r="N119" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O119" s="8" t="s">
+        <v>1126</v>
+      </c>
+      <c r="P119" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q119" s="8" t="s">
+        <v>1127</v>
+      </c>
+      <c r="R119" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S119" s="8" t="s">
+        <v>1128</v>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" s="15"/>
-      <c r="B120" s="16"/>
-      <c r="C120" s="16"/>
-      <c r="D120" s="16"/>
-      <c r="E120" s="11"/>
-      <c r="F120" s="11"/>
-      <c r="G120" s="16"/>
-      <c r="H120" s="16"/>
-      <c r="I120" s="11"/>
-      <c r="J120" s="11"/>
-      <c r="K120" s="11"/>
-      <c r="L120" s="16"/>
-      <c r="M120" s="11"/>
-      <c r="N120" s="11"/>
-      <c r="O120" s="11"/>
-      <c r="P120" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q120" s="11"/>
-      <c r="R120" s="11"/>
-      <c r="S120" s="11"/>
+      <c r="A120" s="4" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C120" s="7" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D120" s="7" t="s">
+        <v>1131</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>1132</v>
+      </c>
+      <c r="F120" s="8" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G120" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H120" s="13" t="s">
+        <v>1133</v>
+      </c>
+      <c r="I120" s="14">
+        <v>46127.0</v>
+      </c>
+      <c r="J120" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K120" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L120" s="7" t="s">
+        <v>1009</v>
+      </c>
+      <c r="M120" s="8" t="s">
+        <v>1134</v>
+      </c>
+      <c r="N120" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O120" s="8" t="s">
+        <v>1135</v>
+      </c>
+      <c r="P120" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q120" s="8" t="s">
+        <v>1136</v>
+      </c>
+      <c r="R120" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S120" s="8" t="s">
+        <v>1137</v>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" s="15"/>
-      <c r="B121" s="16"/>
-      <c r="C121" s="16"/>
-      <c r="D121" s="16"/>
-      <c r="E121" s="11"/>
-      <c r="F121" s="11"/>
-      <c r="G121" s="16"/>
-      <c r="H121" s="16"/>
-      <c r="I121" s="11"/>
-      <c r="J121" s="11"/>
-      <c r="K121" s="11"/>
-      <c r="L121" s="16"/>
-      <c r="M121" s="11"/>
-      <c r="N121" s="11"/>
-      <c r="O121" s="11"/>
-      <c r="P121" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q121" s="11"/>
-      <c r="R121" s="11"/>
-      <c r="S121" s="11"/>
+      <c r="A121" s="4" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C121" s="7" t="s">
+        <v>1140</v>
+      </c>
+      <c r="D121" s="7" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E121" s="8" t="s">
+        <v>1142</v>
+      </c>
+      <c r="F121" s="8" t="s">
+        <v>1143</v>
+      </c>
+      <c r="G121" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H121" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I121" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="J121" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K121" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L121" s="7" t="s">
+        <v>1144</v>
+      </c>
+      <c r="M121" s="8" t="s">
+        <v>1145</v>
+      </c>
+      <c r="N121" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O121" s="8" t="s">
+        <v>1146</v>
+      </c>
+      <c r="P121" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q121" s="8" t="s">
+        <v>1147</v>
+      </c>
+      <c r="R121" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S121" s="8" t="s">
+        <v>1148</v>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" s="15"/>
-      <c r="B122" s="16"/>
-      <c r="C122" s="16"/>
-      <c r="D122" s="16"/>
-      <c r="E122" s="11"/>
-      <c r="F122" s="11"/>
-      <c r="G122" s="16"/>
-      <c r="H122" s="16"/>
-      <c r="I122" s="11"/>
-      <c r="J122" s="11"/>
-      <c r="K122" s="11"/>
-      <c r="L122" s="16"/>
-      <c r="M122" s="11"/>
-      <c r="N122" s="11"/>
-      <c r="O122" s="11"/>
-      <c r="P122" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q122" s="11"/>
-      <c r="R122" s="11"/>
-      <c r="S122" s="11"/>
+      <c r="A122" s="4" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D122" s="7" t="s">
+        <v>1151</v>
+      </c>
+      <c r="E122" s="8" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F122" s="8" t="s">
+        <v>1143</v>
+      </c>
+      <c r="G122" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H122" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I122" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="J122" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K122" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L122" s="7" t="s">
+        <v>1144</v>
+      </c>
+      <c r="M122" s="8" t="s">
+        <v>1153</v>
+      </c>
+      <c r="N122" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O122" s="8" t="s">
+        <v>1154</v>
+      </c>
+      <c r="P122" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q122" s="8" t="s">
+        <v>1155</v>
+      </c>
+      <c r="R122" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S122" s="8" t="s">
+        <v>1156</v>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="15"/>
-      <c r="B123" s="16"/>
-      <c r="C123" s="16"/>
-      <c r="D123" s="16"/>
-      <c r="E123" s="11"/>
-      <c r="F123" s="11"/>
-      <c r="G123" s="16"/>
-      <c r="H123" s="16"/>
-      <c r="I123" s="11"/>
-      <c r="J123" s="11"/>
-      <c r="K123" s="11"/>
-      <c r="L123" s="16"/>
-      <c r="M123" s="11"/>
-      <c r="N123" s="11"/>
-      <c r="O123" s="11"/>
-      <c r="P123" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q123" s="11"/>
-      <c r="R123" s="11"/>
-      <c r="S123" s="11"/>
+      <c r="A123" s="4" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C123" s="7" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D123" s="7" t="s">
+        <v>1159</v>
+      </c>
+      <c r="E123" s="8" t="s">
+        <v>1160</v>
+      </c>
+      <c r="F123" s="8" t="s">
+        <v>1161</v>
+      </c>
+      <c r="G123" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H123" s="13" t="s">
+        <v>1080</v>
+      </c>
+      <c r="I123" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="J123" s="14">
+        <v>46199.0</v>
+      </c>
+      <c r="K123" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="L123" s="7" t="s">
+        <v>1162</v>
+      </c>
+      <c r="M123" s="8" t="s">
+        <v>1163</v>
+      </c>
+      <c r="N123" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="O123" s="8" t="s">
+        <v>1164</v>
+      </c>
+      <c r="P123" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q123" s="8" t="s">
+        <v>1165</v>
+      </c>
+      <c r="R123" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="S123" s="8" t="s">
+        <v>1166</v>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" s="15"/>
-      <c r="B124" s="16"/>
-      <c r="C124" s="16"/>
-      <c r="D124" s="16"/>
-      <c r="E124" s="11"/>
-      <c r="F124" s="11"/>
-      <c r="G124" s="16"/>
-      <c r="H124" s="16"/>
-      <c r="I124" s="11"/>
-      <c r="J124" s="11"/>
-      <c r="K124" s="11"/>
-      <c r="L124" s="16"/>
-      <c r="M124" s="11"/>
-      <c r="N124" s="11"/>
-      <c r="O124" s="11"/>
-      <c r="P124" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q124" s="11"/>
-      <c r="R124" s="11"/>
-      <c r="S124" s="11"/>
+      <c r="A124" s="4" t="s">
+        <v>1167</v>
+      </c>
+      <c r="B124" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C124" s="7" t="s">
+        <v>1168</v>
+      </c>
+      <c r="D124" s="7" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E124" s="8" t="s">
+        <v>1170</v>
+      </c>
+      <c r="F124" s="8" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G124" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="H124" s="13" t="s">
+        <v>1172</v>
+      </c>
+      <c r="I124" s="14">
+        <v>46191.0</v>
+      </c>
+      <c r="J124" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K124" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L124" s="7" t="s">
+        <v>1174</v>
+      </c>
+      <c r="M124" s="8" t="s">
+        <v>1175</v>
+      </c>
+      <c r="N124" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O124" s="8" t="s">
+        <v>1176</v>
+      </c>
+      <c r="P124" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q124" s="8" t="s">
+        <v>1177</v>
+      </c>
+      <c r="R124" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S124" s="8" t="s">
+        <v>1178</v>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="15"/>
-      <c r="B125" s="16"/>
-      <c r="C125" s="16"/>
-      <c r="D125" s="16"/>
-      <c r="E125" s="11"/>
-      <c r="F125" s="11"/>
-      <c r="G125" s="16"/>
-      <c r="H125" s="16"/>
-      <c r="I125" s="11"/>
-      <c r="J125" s="11"/>
-      <c r="K125" s="11"/>
-      <c r="L125" s="16"/>
-      <c r="M125" s="11"/>
-      <c r="N125" s="11"/>
-      <c r="O125" s="11"/>
-      <c r="P125" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q125" s="11"/>
-      <c r="R125" s="11"/>
-      <c r="S125" s="11"/>
+      <c r="A125" s="4" t="s">
+        <v>1179</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C125" s="7" t="s">
+        <v>1181</v>
+      </c>
+      <c r="D125" s="7" t="s">
+        <v>1182</v>
+      </c>
+      <c r="E125" s="8" t="s">
+        <v>1183</v>
+      </c>
+      <c r="F125" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G125" s="7" t="s">
+        <v>1185</v>
+      </c>
+      <c r="H125" s="13" t="s">
+        <v>1186</v>
+      </c>
+      <c r="I125" s="14">
+        <v>46191.0</v>
+      </c>
+      <c r="J125" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K125" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L125" s="7" t="s">
+        <v>1187</v>
+      </c>
+      <c r="M125" s="8" t="s">
+        <v>1188</v>
+      </c>
+      <c r="N125" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="O125" s="8" t="s">
+        <v>1189</v>
+      </c>
+      <c r="P125" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q125" s="8" t="s">
+        <v>1190</v>
+      </c>
+      <c r="R125" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="S125" s="8" t="s">
+        <v>1191</v>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" s="15"/>
-      <c r="B126" s="16"/>
-      <c r="C126" s="16"/>
-      <c r="D126" s="16"/>
-      <c r="E126" s="11"/>
-      <c r="F126" s="11"/>
-      <c r="G126" s="16"/>
-      <c r="H126" s="16"/>
-      <c r="I126" s="11"/>
-      <c r="J126" s="11"/>
-      <c r="K126" s="11"/>
-      <c r="L126" s="16"/>
-      <c r="M126" s="11"/>
-      <c r="N126" s="11"/>
-      <c r="O126" s="11"/>
-      <c r="P126" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q126" s="11"/>
-      <c r="R126" s="11"/>
-      <c r="S126" s="11"/>
+      <c r="A126" s="4" t="s">
+        <v>1192</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="C126" s="7" t="s">
+        <v>1193</v>
+      </c>
+      <c r="D126" s="7" t="s">
+        <v>1194</v>
+      </c>
+      <c r="E126" s="8" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F126" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G126" s="7" t="s">
+        <v>1196</v>
+      </c>
+      <c r="H126" s="7" t="s">
+        <v>1197</v>
+      </c>
+      <c r="I126" s="14">
+        <v>46191.0</v>
+      </c>
+      <c r="J126" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K126" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L126" s="7" t="s">
+        <v>1198</v>
+      </c>
+      <c r="M126" s="8" t="s">
+        <v>1199</v>
+      </c>
+      <c r="N126" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O126" s="8" t="s">
+        <v>1200</v>
+      </c>
+      <c r="P126" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q126" s="8" t="s">
+        <v>1201</v>
+      </c>
+      <c r="R126" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S126" s="8" t="s">
+        <v>1202</v>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="15"/>
-      <c r="B127" s="16"/>
-      <c r="C127" s="16"/>
-      <c r="D127" s="16"/>
-      <c r="E127" s="11"/>
-      <c r="F127" s="11"/>
-      <c r="G127" s="16"/>
-      <c r="H127" s="16"/>
-      <c r="I127" s="11"/>
-      <c r="J127" s="11"/>
-      <c r="K127" s="11"/>
-      <c r="L127" s="16"/>
-      <c r="M127" s="11"/>
-      <c r="N127" s="11"/>
-      <c r="O127" s="11"/>
-      <c r="P127" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q127" s="11"/>
-      <c r="R127" s="11"/>
-      <c r="S127" s="11"/>
+      <c r="A127" s="4" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C127" s="7" t="s">
+        <v>1204</v>
+      </c>
+      <c r="D127" s="7" t="s">
+        <v>1205</v>
+      </c>
+      <c r="E127" s="8" t="s">
+        <v>1206</v>
+      </c>
+      <c r="F127" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G127" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="H127" s="7" t="s">
+        <v>1207</v>
+      </c>
+      <c r="I127" s="14">
+        <v>46191.0</v>
+      </c>
+      <c r="J127" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K127" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L127" s="7" t="s">
+        <v>1208</v>
+      </c>
+      <c r="M127" s="8" t="s">
+        <v>1209</v>
+      </c>
+      <c r="N127" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="O127" s="8" t="s">
+        <v>1210</v>
+      </c>
+      <c r="P127" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q127" s="8" t="s">
+        <v>1211</v>
+      </c>
+      <c r="R127" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="S127" s="8" t="s">
+        <v>1212</v>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" s="15"/>
-      <c r="B128" s="16"/>
-      <c r="C128" s="16"/>
-      <c r="D128" s="16"/>
-      <c r="E128" s="11"/>
-      <c r="F128" s="11"/>
-      <c r="G128" s="16"/>
-      <c r="H128" s="16"/>
-      <c r="I128" s="11"/>
-      <c r="J128" s="11"/>
-      <c r="K128" s="11"/>
-      <c r="L128" s="16"/>
-      <c r="M128" s="11"/>
-      <c r="N128" s="11"/>
-      <c r="O128" s="11"/>
-      <c r="P128" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q128" s="11"/>
-      <c r="R128" s="11"/>
-      <c r="S128" s="11"/>
+      <c r="A128" s="4" t="s">
+        <v>1213</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C128" s="7" t="s">
+        <v>1214</v>
+      </c>
+      <c r="D128" s="7" t="s">
+        <v>1215</v>
+      </c>
+      <c r="E128" s="8" t="s">
+        <v>1216</v>
+      </c>
+      <c r="F128" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G128" s="7" t="s">
+        <v>1217</v>
+      </c>
+      <c r="H128" s="7" t="s">
+        <v>1218</v>
+      </c>
+      <c r="I128" s="14">
+        <v>46191.0</v>
+      </c>
+      <c r="J128" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K128" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L128" s="7" t="s">
+        <v>1219</v>
+      </c>
+      <c r="M128" s="8" t="s">
+        <v>1220</v>
+      </c>
+      <c r="N128" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="O128" s="8" t="s">
+        <v>1221</v>
+      </c>
+      <c r="P128" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q128" s="8" t="s">
+        <v>1222</v>
+      </c>
+      <c r="R128" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="S128" s="8" t="s">
+        <v>1223</v>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="15"/>
-      <c r="B129" s="16"/>
-      <c r="C129" s="16"/>
-      <c r="D129" s="16"/>
-      <c r="E129" s="11"/>
-      <c r="F129" s="11"/>
-      <c r="G129" s="16"/>
-      <c r="H129" s="16"/>
-      <c r="I129" s="11"/>
-      <c r="J129" s="11"/>
-      <c r="K129" s="11"/>
-      <c r="L129" s="16"/>
-      <c r="M129" s="11"/>
-      <c r="N129" s="11"/>
-      <c r="O129" s="11"/>
-      <c r="P129" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q129" s="11"/>
-      <c r="R129" s="11"/>
-      <c r="S129" s="11"/>
+      <c r="A129" s="4" t="s">
+        <v>1224</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C129" s="7" t="s">
+        <v>1225</v>
+      </c>
+      <c r="D129" s="7" t="s">
+        <v>1226</v>
+      </c>
+      <c r="E129" s="8" t="s">
+        <v>1227</v>
+      </c>
+      <c r="F129" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G129" s="7" t="s">
+        <v>1228</v>
+      </c>
+      <c r="H129" s="7" t="s">
+        <v>1229</v>
+      </c>
+      <c r="I129" s="14">
+        <v>46191.0</v>
+      </c>
+      <c r="J129" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K129" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L129" s="7" t="s">
+        <v>1230</v>
+      </c>
+      <c r="M129" s="8" t="s">
+        <v>1231</v>
+      </c>
+      <c r="N129" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O129" s="8" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P129" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q129" s="8" t="s">
+        <v>1233</v>
+      </c>
+      <c r="R129" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S129" s="8" t="s">
+        <v>1234</v>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="15"/>
-      <c r="B130" s="16"/>
-      <c r="C130" s="16"/>
-      <c r="D130" s="16"/>
-      <c r="E130" s="11"/>
-      <c r="F130" s="11"/>
-      <c r="G130" s="16"/>
-      <c r="H130" s="16"/>
-      <c r="I130" s="11"/>
-      <c r="J130" s="11"/>
-      <c r="K130" s="11"/>
-      <c r="L130" s="16"/>
-      <c r="M130" s="11"/>
-      <c r="N130" s="11"/>
-      <c r="O130" s="11"/>
-      <c r="P130" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q130" s="11"/>
-      <c r="R130" s="11"/>
-      <c r="S130" s="11"/>
+      <c r="A130" s="4" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="C130" s="7" t="s">
+        <v>1236</v>
+      </c>
+      <c r="D130" s="7" t="s">
+        <v>1237</v>
+      </c>
+      <c r="E130" s="8" t="s">
+        <v>1238</v>
+      </c>
+      <c r="F130" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G130" s="7" t="s">
+        <v>1239</v>
+      </c>
+      <c r="H130" s="13" t="s">
+        <v>1240</v>
+      </c>
+      <c r="I130" s="14">
+        <v>46191.0</v>
+      </c>
+      <c r="J130" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K130" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L130" s="7" t="s">
+        <v>1241</v>
+      </c>
+      <c r="M130" s="8" t="s">
+        <v>1242</v>
+      </c>
+      <c r="N130" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="O130" s="8" t="s">
+        <v>1243</v>
+      </c>
+      <c r="P130" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q130" s="8" t="s">
+        <v>1244</v>
+      </c>
+      <c r="R130" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S130" s="8" t="s">
+        <v>1245</v>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="15"/>
-      <c r="B131" s="16"/>
-      <c r="C131" s="16"/>
-      <c r="D131" s="16"/>
-      <c r="E131" s="11"/>
-      <c r="F131" s="11"/>
-      <c r="G131" s="16"/>
-      <c r="H131" s="16"/>
-      <c r="I131" s="11"/>
-      <c r="J131" s="11"/>
-      <c r="K131" s="11"/>
-      <c r="L131" s="16"/>
-      <c r="M131" s="11"/>
-      <c r="N131" s="11"/>
-      <c r="O131" s="11"/>
-      <c r="P131" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q131" s="11"/>
-      <c r="R131" s="11"/>
-      <c r="S131" s="11"/>
+      <c r="A131" s="4" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="C131" s="7" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D131" s="7" t="s">
+        <v>1248</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>1249</v>
+      </c>
+      <c r="F131" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G131" s="7" t="s">
+        <v>1250</v>
+      </c>
+      <c r="H131" s="7" t="s">
+        <v>1251</v>
+      </c>
+      <c r="I131" s="14">
+        <v>46192.0</v>
+      </c>
+      <c r="J131" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K131" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L131" s="7" t="s">
+        <v>1252</v>
+      </c>
+      <c r="M131" s="8" t="s">
+        <v>1253</v>
+      </c>
+      <c r="N131" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="O131" s="8" t="s">
+        <v>1254</v>
+      </c>
+      <c r="P131" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q131" s="8" t="s">
+        <v>1255</v>
+      </c>
+      <c r="R131" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S131" s="8" t="s">
+        <v>1256</v>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="15"/>
-      <c r="B132" s="16"/>
-      <c r="C132" s="16"/>
-      <c r="D132" s="16"/>
-      <c r="E132" s="11"/>
-      <c r="F132" s="11"/>
-      <c r="G132" s="16"/>
-      <c r="H132" s="16"/>
-      <c r="I132" s="11"/>
-      <c r="J132" s="11"/>
-      <c r="K132" s="11"/>
-      <c r="L132" s="16"/>
-      <c r="M132" s="11"/>
-      <c r="N132" s="11"/>
-      <c r="O132" s="11"/>
-      <c r="P132" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q132" s="11"/>
-      <c r="R132" s="11"/>
-      <c r="S132" s="11"/>
+      <c r="A132" s="4" t="s">
+        <v>1257</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C132" s="7" t="s">
+        <v>1258</v>
+      </c>
+      <c r="D132" s="7" t="s">
+        <v>1259</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>1260</v>
+      </c>
+      <c r="F132" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G132" s="7" t="s">
+        <v>1261</v>
+      </c>
+      <c r="H132" s="7" t="s">
+        <v>1262</v>
+      </c>
+      <c r="I132" s="14">
+        <v>46192.0</v>
+      </c>
+      <c r="J132" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K132" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L132" s="7" t="s">
+        <v>1263</v>
+      </c>
+      <c r="M132" s="8" t="s">
+        <v>1264</v>
+      </c>
+      <c r="N132" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="O132" s="8" t="s">
+        <v>1265</v>
+      </c>
+      <c r="P132" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q132" s="8" t="s">
+        <v>1266</v>
+      </c>
+      <c r="R132" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="S132" s="8" t="s">
+        <v>1267</v>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="15"/>
-      <c r="B133" s="16"/>
-      <c r="C133" s="16"/>
-      <c r="D133" s="16"/>
-      <c r="E133" s="11"/>
-      <c r="F133" s="11"/>
-      <c r="G133" s="16"/>
-      <c r="H133" s="16"/>
-      <c r="I133" s="11"/>
-      <c r="J133" s="11"/>
-      <c r="K133" s="11"/>
-      <c r="L133" s="16"/>
-      <c r="M133" s="11"/>
-      <c r="N133" s="11"/>
-      <c r="O133" s="11"/>
-      <c r="P133" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q133" s="11"/>
-      <c r="R133" s="11"/>
-      <c r="S133" s="11"/>
+      <c r="A133" s="4" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C133" s="7" t="s">
+        <v>1269</v>
+      </c>
+      <c r="D133" s="7" t="s">
+        <v>1270</v>
+      </c>
+      <c r="E133" s="8" t="s">
+        <v>1271</v>
+      </c>
+      <c r="F133" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G133" s="7" t="s">
+        <v>1272</v>
+      </c>
+      <c r="H133" s="13" t="s">
+        <v>1273</v>
+      </c>
+      <c r="I133" s="14">
+        <v>46191.0</v>
+      </c>
+      <c r="J133" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K133" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L133" s="7" t="s">
+        <v>1274</v>
+      </c>
+      <c r="M133" s="8" t="s">
+        <v>1275</v>
+      </c>
+      <c r="N133" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="O133" s="8" t="s">
+        <v>1276</v>
+      </c>
+      <c r="P133" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q133" s="8" t="s">
+        <v>1277</v>
+      </c>
+      <c r="R133" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S133" s="8" t="s">
+        <v>1278</v>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="15"/>
-      <c r="B134" s="16"/>
-      <c r="C134" s="16"/>
-      <c r="D134" s="16"/>
-      <c r="E134" s="11"/>
-      <c r="F134" s="11"/>
-      <c r="G134" s="16"/>
-      <c r="H134" s="16"/>
-      <c r="I134" s="11"/>
-      <c r="J134" s="11"/>
-      <c r="K134" s="11"/>
-      <c r="L134" s="16"/>
-      <c r="M134" s="11"/>
-      <c r="N134" s="11"/>
-      <c r="O134" s="11"/>
-      <c r="P134" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q134" s="11"/>
-      <c r="R134" s="11"/>
-      <c r="S134" s="11"/>
+      <c r="A134" s="4" t="s">
+        <v>1279</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C134" s="7" t="s">
+        <v>1280</v>
+      </c>
+      <c r="D134" s="7" t="s">
+        <v>1281</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>1282</v>
+      </c>
+      <c r="F134" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G134" s="7" t="s">
+        <v>1283</v>
+      </c>
+      <c r="H134" s="13" t="s">
+        <v>1284</v>
+      </c>
+      <c r="I134" s="14">
+        <v>46194.0</v>
+      </c>
+      <c r="J134" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K134" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L134" s="7" t="s">
+        <v>1285</v>
+      </c>
+      <c r="M134" s="8" t="s">
+        <v>1286</v>
+      </c>
+      <c r="N134" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="O134" s="8" t="s">
+        <v>1287</v>
+      </c>
+      <c r="P134" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q134" s="8" t="s">
+        <v>1288</v>
+      </c>
+      <c r="R134" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S134" s="8" t="s">
+        <v>1289</v>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" s="15"/>
-      <c r="B135" s="16"/>
-      <c r="C135" s="16"/>
-      <c r="D135" s="16"/>
-      <c r="E135" s="11"/>
-      <c r="F135" s="11"/>
-      <c r="G135" s="16"/>
-      <c r="H135" s="16"/>
-      <c r="I135" s="11"/>
-      <c r="J135" s="11"/>
-      <c r="K135" s="11"/>
-      <c r="L135" s="16"/>
-      <c r="M135" s="11"/>
-      <c r="N135" s="11"/>
-      <c r="O135" s="11"/>
-      <c r="P135" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q135" s="11"/>
-      <c r="R135" s="11"/>
-      <c r="S135" s="11"/>
+      <c r="A135" s="4" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C135" s="7" t="s">
+        <v>1291</v>
+      </c>
+      <c r="D135" s="7" t="s">
+        <v>1292</v>
+      </c>
+      <c r="E135" s="8" t="s">
+        <v>1293</v>
+      </c>
+      <c r="F135" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G135" s="7" t="s">
+        <v>1294</v>
+      </c>
+      <c r="H135" s="7" t="s">
+        <v>1295</v>
+      </c>
+      <c r="I135" s="14">
+        <v>46194.0</v>
+      </c>
+      <c r="J135" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K135" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L135" s="7" t="s">
+        <v>1296</v>
+      </c>
+      <c r="M135" s="8" t="s">
+        <v>1297</v>
+      </c>
+      <c r="N135" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O135" s="8" t="s">
+        <v>1298</v>
+      </c>
+      <c r="P135" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q135" s="8" t="s">
+        <v>1299</v>
+      </c>
+      <c r="R135" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S135" s="8" t="s">
+        <v>1300</v>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" s="15"/>
-      <c r="B136" s="16"/>
-      <c r="C136" s="16"/>
-      <c r="D136" s="16"/>
-      <c r="E136" s="11"/>
-      <c r="F136" s="11"/>
-      <c r="G136" s="16"/>
-      <c r="H136" s="16"/>
-      <c r="I136" s="11"/>
-      <c r="J136" s="11"/>
-      <c r="K136" s="11"/>
-      <c r="L136" s="16"/>
-      <c r="M136" s="11"/>
-      <c r="N136" s="11"/>
-      <c r="O136" s="11"/>
-      <c r="P136" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q136" s="11"/>
-      <c r="R136" s="11"/>
-      <c r="S136" s="11"/>
+      <c r="A136" s="4" t="s">
+        <v>1301</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="C136" s="7" t="s">
+        <v>1302</v>
+      </c>
+      <c r="D136" s="7" t="s">
+        <v>1303</v>
+      </c>
+      <c r="E136" s="8" t="s">
+        <v>1304</v>
+      </c>
+      <c r="F136" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G136" s="7" t="s">
+        <v>1283</v>
+      </c>
+      <c r="H136" s="7" t="s">
+        <v>1305</v>
+      </c>
+      <c r="I136" s="14">
+        <v>46194.0</v>
+      </c>
+      <c r="J136" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K136" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L136" s="7" t="s">
+        <v>1306</v>
+      </c>
+      <c r="M136" s="8" t="s">
+        <v>1307</v>
+      </c>
+      <c r="N136" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="O136" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="P136" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q136" s="8" t="s">
+        <v>1309</v>
+      </c>
+      <c r="R136" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="S136" s="8" t="s">
+        <v>1310</v>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" s="15"/>
-      <c r="B137" s="16"/>
-      <c r="C137" s="16"/>
-      <c r="D137" s="16"/>
-      <c r="E137" s="11"/>
-      <c r="F137" s="11"/>
-      <c r="G137" s="16"/>
-      <c r="H137" s="16"/>
-      <c r="I137" s="11"/>
-      <c r="J137" s="11"/>
-      <c r="K137" s="11"/>
-      <c r="L137" s="16"/>
-      <c r="M137" s="11"/>
-      <c r="N137" s="11"/>
-      <c r="O137" s="11"/>
-      <c r="P137" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q137" s="11"/>
-      <c r="R137" s="11"/>
-      <c r="S137" s="11"/>
+      <c r="A137" s="4" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B137" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="C137" s="7" t="s">
+        <v>1312</v>
+      </c>
+      <c r="D137" s="7" t="s">
+        <v>1313</v>
+      </c>
+      <c r="E137" s="8" t="s">
+        <v>1314</v>
+      </c>
+      <c r="F137" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G137" s="7" t="s">
+        <v>1283</v>
+      </c>
+      <c r="H137" s="13" t="s">
+        <v>1315</v>
+      </c>
+      <c r="I137" s="14">
+        <v>46194.0</v>
+      </c>
+      <c r="J137" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K137" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L137" s="7" t="s">
+        <v>540</v>
+      </c>
+      <c r="M137" s="8" t="s">
+        <v>1316</v>
+      </c>
+      <c r="N137" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O137" s="8" t="s">
+        <v>1317</v>
+      </c>
+      <c r="P137" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q137" s="8" t="s">
+        <v>1318</v>
+      </c>
+      <c r="R137" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="S137" s="8" t="s">
+        <v>1319</v>
+      </c>
     </row>
     <row r="138">
-      <c r="A138" s="15"/>
-      <c r="B138" s="16"/>
-      <c r="C138" s="16"/>
-      <c r="D138" s="16"/>
-      <c r="E138" s="11"/>
-      <c r="F138" s="11"/>
-      <c r="G138" s="16"/>
-      <c r="H138" s="16"/>
-      <c r="I138" s="11"/>
-      <c r="J138" s="11"/>
-      <c r="K138" s="11"/>
-      <c r="L138" s="16"/>
-      <c r="M138" s="11"/>
-      <c r="N138" s="11"/>
-      <c r="O138" s="11"/>
-      <c r="P138" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q138" s="11"/>
-      <c r="R138" s="11"/>
-      <c r="S138" s="11"/>
+      <c r="A138" s="4" t="s">
+        <v>1320</v>
+      </c>
+      <c r="B138" s="5" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C138" s="7" t="s">
+        <v>1321</v>
+      </c>
+      <c r="D138" s="7" t="s">
+        <v>1322</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>1323</v>
+      </c>
+      <c r="F138" s="8" t="s">
+        <v>1184</v>
+      </c>
+      <c r="G138" s="7" t="s">
+        <v>1324</v>
+      </c>
+      <c r="H138" s="7" t="s">
+        <v>1325</v>
+      </c>
+      <c r="I138" s="14">
+        <v>46198.0</v>
+      </c>
+      <c r="J138" s="14">
+        <v>46200.0</v>
+      </c>
+      <c r="K138" s="8" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L138" s="7" t="s">
+        <v>1326</v>
+      </c>
+      <c r="M138" s="8" t="s">
+        <v>1327</v>
+      </c>
+      <c r="N138" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="O138" s="8" t="s">
+        <v>1328</v>
+      </c>
+      <c r="P138" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q138" s="8" t="s">
+        <v>1329</v>
+      </c>
+      <c r="R138" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="S138" s="8" t="s">
+        <v>1330</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="15"/>
@@ -10512,25 +12855,27 @@
       <c r="S140" s="11"/>
     </row>
     <row r="141">
-      <c r="A141" s="4"/>
-      <c r="B141" s="5"/>
-      <c r="C141" s="7"/>
-      <c r="D141" s="7"/>
-      <c r="E141" s="8"/>
-      <c r="F141" s="8"/>
-      <c r="G141" s="7"/>
-      <c r="H141" s="7"/>
-      <c r="I141" s="8"/>
-      <c r="J141" s="8"/>
-      <c r="K141" s="8"/>
-      <c r="L141" s="5"/>
-      <c r="M141" s="8"/>
-      <c r="N141" s="8"/>
-      <c r="O141" s="8"/>
-      <c r="P141" s="8"/>
-      <c r="Q141" s="8"/>
-      <c r="R141" s="8"/>
-      <c r="S141" s="8"/>
+      <c r="A141" s="15"/>
+      <c r="B141" s="16"/>
+      <c r="C141" s="16"/>
+      <c r="D141" s="16"/>
+      <c r="E141" s="11"/>
+      <c r="F141" s="11"/>
+      <c r="G141" s="16"/>
+      <c r="H141" s="16"/>
+      <c r="I141" s="11"/>
+      <c r="J141" s="11"/>
+      <c r="K141" s="11"/>
+      <c r="L141" s="16"/>
+      <c r="M141" s="11"/>
+      <c r="N141" s="11"/>
+      <c r="O141" s="11"/>
+      <c r="P141" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q141" s="11"/>
+      <c r="R141" s="11"/>
+      <c r="S141" s="11"/>
     </row>
     <row r="142">
       <c r="A142" s="15"/>
@@ -29852,87 +32197,18 @@
       <c r="R981" s="11"/>
       <c r="S981" s="11"/>
     </row>
-    <row r="982">
-      <c r="A982" s="15"/>
-      <c r="B982" s="16"/>
-      <c r="C982" s="16"/>
-      <c r="D982" s="16"/>
-      <c r="E982" s="11"/>
-      <c r="F982" s="11"/>
-      <c r="G982" s="16"/>
-      <c r="H982" s="16"/>
-      <c r="I982" s="11"/>
-      <c r="J982" s="11"/>
-      <c r="K982" s="11"/>
-      <c r="L982" s="16"/>
-      <c r="M982" s="11"/>
-      <c r="N982" s="11"/>
-      <c r="O982" s="11"/>
-      <c r="P982" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q982" s="11"/>
-      <c r="R982" s="11"/>
-      <c r="S982" s="11"/>
-    </row>
-    <row r="983">
-      <c r="A983" s="15"/>
-      <c r="B983" s="16"/>
-      <c r="C983" s="16"/>
-      <c r="D983" s="16"/>
-      <c r="E983" s="11"/>
-      <c r="F983" s="11"/>
-      <c r="G983" s="16"/>
-      <c r="H983" s="16"/>
-      <c r="I983" s="11"/>
-      <c r="J983" s="11"/>
-      <c r="K983" s="11"/>
-      <c r="L983" s="16"/>
-      <c r="M983" s="11"/>
-      <c r="N983" s="11"/>
-      <c r="O983" s="11"/>
-      <c r="P983" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q983" s="11"/>
-      <c r="R983" s="11"/>
-      <c r="S983" s="11"/>
-    </row>
-    <row r="984">
-      <c r="A984" s="15"/>
-      <c r="B984" s="16"/>
-      <c r="C984" s="16"/>
-      <c r="D984" s="16"/>
-      <c r="E984" s="11"/>
-      <c r="F984" s="11"/>
-      <c r="G984" s="16"/>
-      <c r="H984" s="16"/>
-      <c r="I984" s="11"/>
-      <c r="J984" s="11"/>
-      <c r="K984" s="11"/>
-      <c r="L984" s="16"/>
-      <c r="M984" s="11"/>
-      <c r="N984" s="11"/>
-      <c r="O984" s="11"/>
-      <c r="P984" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q984" s="11"/>
-      <c r="R984" s="11"/>
-      <c r="S984" s="11"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B984">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B981">
       <formula1>"Rules,Trades,Resolution,Communication,Other,News,Wallets,Blockchain,Trades"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="R2:R984">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="R2:R981">
       <formula1>"Public,Claimant-Private,Counsel-Only,Attorney review,Internal,Restricted"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N2:N984">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N2:N981">
       <formula1>"Verified,Partially Verified,Unverified,Derived analysis"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:J984">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:J981">
       <formula1>OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D"))</formula1>
     </dataValidation>
   </dataValidations>
@@ -29981,10 +32257,30 @@
     <hyperlink r:id="rId42" ref="H80"/>
     <hyperlink r:id="rId43" ref="S80"/>
     <hyperlink r:id="rId44" ref="S84"/>
+    <hyperlink r:id="rId45" ref="H105"/>
+    <hyperlink r:id="rId46" ref="H106"/>
+    <hyperlink r:id="rId47" ref="H107"/>
+    <hyperlink r:id="rId48" ref="H108"/>
+    <hyperlink r:id="rId49" ref="H109"/>
+    <hyperlink r:id="rId50" ref="H110"/>
+    <hyperlink r:id="rId51" ref="H111"/>
+    <hyperlink r:id="rId52" ref="H112"/>
+    <hyperlink r:id="rId53" ref="H114"/>
+    <hyperlink r:id="rId54" ref="H117"/>
+    <hyperlink r:id="rId55" ref="H118"/>
+    <hyperlink r:id="rId56" ref="H119"/>
+    <hyperlink r:id="rId57" ref="H120"/>
+    <hyperlink r:id="rId58" ref="H123"/>
+    <hyperlink r:id="rId59" ref="H124"/>
+    <hyperlink r:id="rId60" ref="H125"/>
+    <hyperlink r:id="rId61" ref="H130"/>
+    <hyperlink r:id="rId62" ref="H133"/>
+    <hyperlink r:id="rId63" ref="H134"/>
+    <hyperlink r:id="rId64" ref="H137"/>
   </hyperlinks>
-  <drawing r:id="rId45"/>
+  <drawing r:id="rId65"/>
   <tableParts count="1">
-    <tablePart r:id="rId47"/>
+    <tablePart r:id="rId67"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>